<commit_message>
Initial commit: Rubis offline-first audit tool
Features:
- Dual AI strategy (OpenAI + Ollama local)
- Automated setup scripts (install-ollama.ps1, start-rubis.ps1)
- 100% offline operation after initial setup
- Complete audit workflow (5 phases + sprint 1)
- Dashboard with KPIs and conformity matrix
- Export capabilities (CSV, DOCX, Markdown)
- Audit logging and tracking
- Question generation from referential (PDF/Excel)

Tech Stack:
- API: Node.js + Fastify + lowdb
- Frontend: React + Vite + TypeScript
- Local persistence: JSON database
- AI: OpenAI API or local Ollama (Mistral 7B Q4)

Documentation:
- GETTING_STARTED.md - Quick start guide
- SETUP_OLLAMA.md - Local AI setup
- SETUP_OPENAI.md - Cloud AI setup
- README.md - Architecture overview
</commit_message>
<xml_diff>
--- a/ROADMAP.xlsx
+++ b/ROADMAP.xlsx
@@ -397,1103 +397,1387 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:I47"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="55.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="70.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="65.83203125" customWidth="1"/>
+    <col min="9" max="9" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>ID</v>
+      </c>
+      <c r="B1" t="str">
         <v>Domaine</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
         <v>Fonctionnalité</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>Description</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>Priorité</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Statut</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
+        <v>Prédécesseurs</v>
+      </c>
+      <c r="H1" t="str">
         <v>Directives d'implémentation</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>Notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>REQ-001</v>
+      </c>
+      <c r="B2" t="str">
         <v>Cœur métier</v>
       </c>
-      <c r="B2" t="str">
+      <c r="C2" t="str">
         <v>Workflow complet d'audit</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>Phase 1.1 Préparation → 1.2 Entretiens → 1.3 Scoring → 1.4 Rapports</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>P0</v>
       </c>
-      <c r="E2" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F2" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G2" t="str">
+        <v>-</v>
+      </c>
+      <c r="H2" t="str">
         <v>Chaque phase est un mode d'affichage séparé dans App.tsx. État global gère la transition.</v>
       </c>
-      <c r="G2" t="str">
+      <c r="I2" t="str">
         <v>MVP complet, testé en production</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>REQ-002</v>
+      </c>
+      <c r="B3" t="str">
         <v>Cœur métier</v>
       </c>
-      <c r="B3" t="str">
+      <c r="C3" t="str">
         <v>Gestion des campagnes d'audit</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>Création, sélection, stockage des campagnes avec métadonnées</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>P0</v>
       </c>
-      <c r="E3" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F3" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G3" t="str">
+        <v>-</v>
+      </c>
+      <c r="H3" t="str">
         <v>Endpoints: POST /campaigns, GET /campaigns. Stockage lowdb en db.data.campaigns</v>
       </c>
-      <c r="G3" t="str">
+      <c r="I3" t="str">
         <v>ID UUID, timestamps, framework (ISO 19011/PASSI)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>REQ-003</v>
+      </c>
+      <c r="B4" t="str">
         <v>Cœur métier</v>
       </c>
-      <c r="B4" t="str">
+      <c r="C4" t="str">
         <v>Gestion des critères d'audit</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>Code, titre, thème pour chaque critère avec lien campagne</v>
       </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <v>P0</v>
       </c>
-      <c r="E4" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F4" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G4" t="str">
+        <v>REQ-002</v>
+      </c>
+      <c r="H4" t="str">
         <v>POST /criteria, GET /criteria?campaignId=. Clé étrangère campaignId.</v>
       </c>
-      <c r="G4" t="str">
+      <c r="I4" t="str">
         <v>Critères liés à campagnes pour isolation des données</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>REQ-004</v>
+      </c>
+      <c r="B5" t="str">
         <v>Cœur métier</v>
       </c>
-      <c r="B5" t="str">
+      <c r="C5" t="str">
         <v>Génération de questions</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>Questions avec text, guidance, theme générées dynamiquement</v>
       </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <v>P0</v>
       </c>
-      <c r="E5" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F5" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G5" t="str">
+        <v>REQ-003</v>
+      </c>
+      <c r="H5" t="str">
         <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
       </c>
-      <c r="G5" t="str">
+      <c r="I5" t="str">
         <v>Peut être depuis template ou IA (voir section IA)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>REQ-005</v>
+      </c>
+      <c r="B6" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B6" t="str">
+      <c r="C6" t="str">
         <v>Génération depuis référentiel</v>
       </c>
-      <c r="C6" t="str">
+      <c r="D6" t="str">
         <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
       </c>
-      <c r="D6" t="str">
-        <v>P1</v>
-      </c>
       <c r="E6" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F6" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G6" t="str">
+        <v>REQ-003</v>
+      </c>
+      <c r="H6" t="str">
         <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
       </c>
-      <c r="G6" t="str">
+      <c r="I6" t="str">
         <v>Limite 50KB texte extrait pour perf API</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>REQ-006</v>
+      </c>
+      <c r="B7" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B7" t="str">
+      <c r="C7" t="str">
         <v>Dual AI strategy - OpenAI</v>
       </c>
-      <c r="C7" t="str">
+      <c r="D7" t="str">
         <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
       </c>
-      <c r="D7" t="str">
-        <v>P1</v>
-      </c>
       <c r="E7" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F7" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G7" t="str">
+        <v>REQ-028</v>
+      </c>
+      <c r="H7" t="str">
         <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
       </c>
-      <c r="G7" t="str">
+      <c r="I7" t="str">
         <v>Fallback si OPENAI_API_KEY absent</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
+        <v>REQ-007</v>
+      </c>
+      <c r="B8" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B8" t="str">
+      <c r="C8" t="str">
         <v>Dual AI strategy - Ollama local</v>
       </c>
-      <c r="C8" t="str">
+      <c r="D8" t="str">
         <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
       </c>
-      <c r="D8" t="str">
-        <v>P1</v>
-      </c>
       <c r="E8" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F8" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G8" t="str">
+        <v>REQ-028</v>
+      </c>
+      <c r="H8" t="str">
         <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
       </c>
-      <c r="G8" t="str">
+      <c r="I8" t="str">
         <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>REQ-008</v>
+      </c>
+      <c r="B9" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B9" t="str">
+      <c r="C9" t="str">
         <v>Model switching UI</v>
       </c>
-      <c r="C9" t="str">
+      <c r="D9" t="str">
         <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
       </c>
-      <c r="D9" t="str">
-        <v>P1</v>
-      </c>
       <c r="E9" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F9" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G9" t="str">
+        <v>REQ-006, REQ-007</v>
+      </c>
+      <c r="H9" t="str">
         <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
       </c>
-      <c r="G9" t="str">
+      <c r="I9" t="str">
         <v>Changement runtime, pas besoin restart API</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
+        <v>REQ-009</v>
+      </c>
+      <c r="B10" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B10" t="str">
+      <c r="C10" t="str">
         <v>Parsing référentiel multi-format</v>
       </c>
-      <c r="C10" t="str">
+      <c r="D10" t="str">
         <v>Support PDF et Excel avec extraction de texte</v>
       </c>
-      <c r="D10" t="str">
-        <v>P1</v>
-      </c>
       <c r="E10" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F10" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G10" t="str">
+        <v>REQ-005</v>
+      </c>
+      <c r="H10" t="str">
         <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
       </c>
-      <c r="G10" t="str">
+      <c r="I10" t="str">
         <v>Gère encodages UTF-8, caractères spéciaux</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
+        <v>REQ-010</v>
+      </c>
+      <c r="B11" t="str">
         <v>IA &amp; Génération</v>
       </c>
-      <c r="B11" t="str">
+      <c r="C11" t="str">
         <v>Prompt dynamique contextuel</v>
       </c>
-      <c r="C11" t="str">
+      <c r="D11" t="str">
         <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
       </c>
-      <c r="D11" t="str">
-        <v>P1</v>
-      </c>
       <c r="E11" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F11" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G11" t="str">
+        <v>REQ-005</v>
+      </c>
+      <c r="H11" t="str">
         <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
       </c>
-      <c r="G11" t="str">
+      <c r="I11" t="str">
         <v>Zod validation sur count (1-10), language (fr/en)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>REQ-011</v>
+      </c>
+      <c r="B12" t="str">
         <v>Structuration données</v>
       </c>
-      <c r="B12" t="str">
+      <c r="C12" t="str">
         <v>Modèle Document</v>
       </c>
-      <c r="C12" t="str">
+      <c r="D12" t="str">
         <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
       </c>
-      <c r="D12" t="str">
+      <c r="E12" t="str">
         <v>P0</v>
       </c>
-      <c r="E12" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F12" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G12" t="str">
+        <v>REQ-002</v>
+      </c>
+      <c r="H12" t="str">
         <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
       </c>
-      <c r="G12" t="str">
+      <c r="I12" t="str">
         <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>REQ-012</v>
+      </c>
+      <c r="B13" t="str">
         <v>Structuration données</v>
       </c>
-      <c r="B13" t="str">
+      <c r="C13" t="str">
         <v>Modèle Interviewé</v>
       </c>
-      <c r="C13" t="str">
+      <c r="D13" t="str">
         <v>Nom complet, rôle, lié à campaign</v>
       </c>
-      <c r="D13" t="str">
+      <c r="E13" t="str">
         <v>P0</v>
       </c>
-      <c r="E13" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F13" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G13" t="str">
+        <v>REQ-002</v>
+      </c>
+      <c r="H13" t="str">
         <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
       </c>
-      <c r="G13" t="str">
+      <c r="I13" t="str">
         <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>REQ-013</v>
+      </c>
+      <c r="B14" t="str">
         <v>Structuration données</v>
       </c>
-      <c r="B14" t="str">
+      <c r="C14" t="str">
         <v>Modèle Note d'entretien</v>
       </c>
-      <c r="C14" t="str">
+      <c r="D14" t="str">
         <v>Contenu libre + scoring, lié à criterion et interviewé</v>
       </c>
-      <c r="D14" t="str">
+      <c r="E14" t="str">
         <v>P0</v>
       </c>
-      <c r="E14" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F14" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G14" t="str">
+        <v>REQ-003, REQ-012</v>
+      </c>
+      <c r="H14" t="str">
         <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
       </c>
-      <c r="G14" t="str">
+      <c r="I14" t="str">
         <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
+        <v>REQ-014</v>
+      </c>
+      <c r="B15" t="str">
         <v>Structuration données</v>
       </c>
-      <c r="B15" t="str">
+      <c r="C15" t="str">
         <v>Matrice de conformité</v>
       </c>
-      <c r="C15" t="str">
+      <c r="D15" t="str">
         <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
       </c>
-      <c r="D15" t="str">
-        <v>P1</v>
-      </c>
       <c r="E15" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F15" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G15" t="str">
+        <v>REQ-013</v>
+      </c>
+      <c r="H15" t="str">
         <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
       </c>
-      <c r="G15" t="str">
+      <c r="I15" t="str">
         <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>REQ-015</v>
+      </c>
+      <c r="B16" t="str">
         <v>Structuration données</v>
       </c>
-      <c r="B16" t="str">
+      <c r="C16" t="str">
         <v>Configuration Métriques</v>
       </c>
-      <c r="C16" t="str">
+      <c r="D16" t="str">
         <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
       </c>
-      <c r="D16" t="str">
-        <v>P1</v>
-      </c>
       <c r="E16" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F16" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G16" t="str">
+        <v>REQ-002</v>
+      </c>
+      <c r="H16" t="str">
         <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
       </c>
-      <c r="G16" t="str">
+      <c r="I16" t="str">
         <v>Format texte (ex: '1-5') pour flexibilité</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v>REQ-016</v>
+      </c>
+      <c r="B17" t="str">
         <v>Audit &amp; Traçabilité</v>
       </c>
-      <c r="B17" t="str">
+      <c r="C17" t="str">
         <v>Audit Log complet</v>
       </c>
-      <c r="C17" t="str">
+      <c r="D17" t="str">
         <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
       </c>
-      <c r="D17" t="str">
-        <v>P1</v>
-      </c>
       <c r="E17" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F17" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G17" t="str">
+        <v>REQ-002, REQ-028</v>
+      </c>
+      <c r="H17" t="str">
         <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
       </c>
-      <c r="G17" t="str">
+      <c r="I17" t="str">
         <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
+        <v>REQ-017</v>
+      </c>
+      <c r="B18" t="str">
         <v>Audit &amp; Traçabilité</v>
       </c>
-      <c r="B18" t="str">
+      <c r="C18" t="str">
         <v>Filtrage logs par période</v>
       </c>
-      <c r="C18" t="str">
+      <c r="D18" t="str">
         <v>Vue 7j, 30j, tout (by date range filter)</v>
       </c>
-      <c r="D18" t="str">
-        <v>P1</v>
-      </c>
       <c r="E18" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F18" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G18" t="str">
+        <v>REQ-016</v>
+      </c>
+      <c r="H18" t="str">
         <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
       </c>
-      <c r="G18" t="str">
+      <c r="I18" t="str">
         <v>Filter UI: dropdown 3 options + affichage dynamique</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v>REQ-018</v>
+      </c>
+      <c r="B19" t="str">
         <v>Audit &amp; Traçabilité</v>
       </c>
-      <c r="B19" t="str">
+      <c r="C19" t="str">
         <v>Filtrage logs par action</v>
       </c>
-      <c r="C19" t="str">
+      <c r="D19" t="str">
         <v>Filter sur type d'action (campaign.created, etc.)</v>
       </c>
-      <c r="D19" t="str">
-        <v>P1</v>
-      </c>
       <c r="E19" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F19" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G19" t="str">
+        <v>REQ-016</v>
+      </c>
+      <c r="H19" t="str">
         <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
       </c>
-      <c r="G19" t="str">
+      <c r="I19" t="str">
         <v>Enum actions découvertes dynamiquement from logs</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
+        <v>REQ-019</v>
+      </c>
+      <c r="B20" t="str">
         <v>Rapports &amp; Exports</v>
       </c>
-      <c r="B20" t="str">
+      <c r="C20" t="str">
         <v>Export DOCX</v>
       </c>
-      <c r="C20" t="str">
+      <c r="D20" t="str">
         <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
       </c>
-      <c r="D20" t="str">
+      <c r="E20" t="str">
         <v>P2</v>
       </c>
-      <c r="E20" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F20" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G20" t="str">
+        <v>REQ-004, REQ-014</v>
+      </c>
+      <c r="H20" t="str">
         <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
       </c>
-      <c r="G20" t="str">
+      <c r="I20" t="str">
         <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>REQ-020</v>
+      </c>
+      <c r="B21" t="str">
         <v>Rapports &amp; Exports</v>
       </c>
-      <c r="B21" t="str">
+      <c r="C21" t="str">
         <v>Export CSV</v>
       </c>
-      <c r="C21" t="str">
+      <c r="D21" t="str">
         <v>Audit logs + conformity matrix en CSV téléchargeable</v>
       </c>
-      <c r="D21" t="str">
+      <c r="E21" t="str">
         <v>P2</v>
       </c>
-      <c r="E21" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F21" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G21" t="str">
+        <v>REQ-014, REQ-016</v>
+      </c>
+      <c r="H21" t="str">
         <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
       </c>
-      <c r="G21" t="str">
+      <c r="I21" t="str">
         <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
+        <v>REQ-021</v>
+      </c>
+      <c r="B22" t="str">
         <v>Rapports &amp; Exports</v>
       </c>
-      <c r="B22" t="str">
+      <c r="C22" t="str">
         <v>Gestion des rapports</v>
       </c>
-      <c r="C22" t="str">
+      <c r="D22" t="str">
         <v>Stocker rapports générés avec titre, date gen, version</v>
       </c>
-      <c r="D22" t="str">
+      <c r="E22" t="str">
         <v>P2</v>
       </c>
-      <c r="E22" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F22" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G22" t="str">
+        <v>REQ-019, REQ-020</v>
+      </c>
+      <c r="H22" t="str">
         <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
       </c>
-      <c r="G22" t="str">
+      <c r="I22" t="str">
         <v>Récupérable dans UI, archivé pour traçabilité</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
+        <v>REQ-022</v>
+      </c>
+      <c r="B23" t="str">
         <v>Dashboard &amp; Visualisation</v>
       </c>
-      <c r="B23" t="str">
+      <c r="C23" t="str">
         <v>KPIs essentiels</v>
       </c>
-      <c r="C23" t="str">
+      <c r="D23" t="str">
         <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
       </c>
-      <c r="D23" t="str">
-        <v>P1</v>
-      </c>
       <c r="E23" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F23" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G23" t="str">
+        <v>REQ-011, REQ-012, REQ-013</v>
+      </c>
+      <c r="H23" t="str">
         <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
       </c>
-      <c r="G23" t="str">
+      <c r="I23" t="str">
         <v>Affiché en gros chiffres zone haute dashboard</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
+        <v>REQ-023</v>
+      </c>
+      <c r="B24" t="str">
         <v>Dashboard &amp; Visualisation</v>
       </c>
-      <c r="B24" t="str">
+      <c r="C24" t="str">
         <v>Matrice de conformité interactive</v>
       </c>
-      <c r="C24" t="str">
+      <c r="D24" t="str">
         <v>Tableau avec % conformité par criterion, tri/filtre</v>
       </c>
-      <c r="D24" t="str">
+      <c r="E24" t="str">
         <v>P2</v>
       </c>
-      <c r="E24" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F24" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G24" t="str">
+        <v>REQ-014</v>
+      </c>
+      <c r="H24" t="str">
         <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
       </c>
-      <c r="G24" t="str">
+      <c r="I24" t="str">
         <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>REQ-024</v>
+      </c>
+      <c r="B25" t="str">
         <v>Dashboard &amp; Visualisation</v>
       </c>
-      <c r="B25" t="str">
+      <c r="C25" t="str">
         <v>Graphiques optionnels (futur)</v>
       </c>
-      <c r="C25" t="str">
+      <c r="D25" t="str">
         <v>Tendances audit timeline, pie charts conformity domains</v>
       </c>
-      <c r="D25" t="str">
+      <c r="E25" t="str">
         <v>P3</v>
       </c>
-      <c r="E25" t="str">
+      <c r="F25" t="str">
         <v>Planifié</v>
       </c>
-      <c r="F25" t="str">
+      <c r="G25" t="str">
+        <v>REQ-022</v>
+      </c>
+      <c r="H25" t="str">
         <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
       </c>
-      <c r="G25" t="str">
+      <c r="I25" t="str">
         <v>MVP n'a pas graphiques, architecture prête pour.</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
+        <v>REQ-025</v>
+      </c>
+      <c r="B26" t="str">
         <v>Configuration &amp; Flexibilité</v>
       </c>
-      <c r="B26" t="str">
+      <c r="C26" t="str">
         <v>Support multilingue</v>
       </c>
-      <c r="C26" t="str">
+      <c r="D26" t="str">
         <v>FR et EN, sélection par campaign</v>
       </c>
-      <c r="D26" t="str">
-        <v>P1</v>
-      </c>
       <c r="E26" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F26" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G26" t="str">
+        <v>REQ-028</v>
+      </c>
+      <c r="H26" t="str">
         <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
       </c>
-      <c r="G26" t="str">
+      <c r="I26" t="str">
         <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
+        <v>REQ-026</v>
+      </c>
+      <c r="B27" t="str">
         <v>Configuration &amp; Flexibilité</v>
       </c>
-      <c r="B27" t="str">
+      <c r="C27" t="str">
         <v>Modèle Ollama configurable</v>
       </c>
-      <c r="C27" t="str">
+      <c r="D27" t="str">
         <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
       </c>
-      <c r="D27" t="str">
-        <v>P1</v>
-      </c>
       <c r="E27" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F27" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G27" t="str">
+        <v>REQ-007</v>
+      </c>
+      <c r="H27" t="str">
         <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
       </c>
-      <c r="G27" t="str">
+      <c r="I27" t="str">
         <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
+        <v>REQ-027</v>
+      </c>
+      <c r="B28" t="str">
         <v>Configuration &amp; Flexibilité</v>
       </c>
-      <c r="B28" t="str">
+      <c r="C28" t="str">
         <v>OpenAI optionnel</v>
       </c>
-      <c r="C28" t="str">
+      <c r="D28" t="str">
         <v>API key via .env, fallback auto Ollama si absent</v>
       </c>
-      <c r="D28" t="str">
-        <v>P1</v>
-      </c>
       <c r="E28" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F28" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G28" t="str">
+        <v>REQ-028</v>
+      </c>
+      <c r="H28" t="str">
         <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
       </c>
-      <c r="G28" t="str">
+      <c r="I28" t="str">
         <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
+        <v>REQ-028</v>
+      </c>
+      <c r="B29" t="str">
         <v>Configuration &amp; Flexibilité</v>
       </c>
-      <c r="B29" t="str">
+      <c r="C29" t="str">
         <v>Thèmes personnalisés</v>
       </c>
-      <c r="C29" t="str">
+      <c r="D29" t="str">
         <v>Texte libre pour documents et questions</v>
       </c>
-      <c r="D29" t="str">
+      <c r="E29" t="str">
         <v>P2</v>
       </c>
-      <c r="E29" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F29" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G29" t="str">
+        <v>-</v>
+      </c>
+      <c r="H29" t="str">
         <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
       </c>
-      <c r="G29" t="str">
+      <c r="I29" t="str">
         <v>Permet flexibilité sur domaines audit custom</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
+        <v>REQ-029</v>
+      </c>
+      <c r="B30" t="str">
         <v>Infrastructure &amp; Déploiement</v>
       </c>
-      <c r="B30" t="str">
+      <c r="C30" t="str">
         <v>Offline-first capability</v>
       </c>
-      <c r="C30" t="str">
+      <c r="D30" t="str">
         <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
       </c>
-      <c r="D30" t="str">
-        <v>P1</v>
-      </c>
       <c r="E30" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F30" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G30" t="str">
+        <v>-</v>
+      </c>
+      <c r="H30" t="str">
         <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
       </c>
-      <c r="G30" t="str">
+      <c r="I30" t="str">
         <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>REQ-030</v>
+      </c>
+      <c r="B31" t="str">
         <v>Infrastructure &amp; Déploiement</v>
       </c>
-      <c r="B31" t="str">
+      <c r="C31" t="str">
         <v>Automation PowerShell</v>
       </c>
-      <c r="C31" t="str">
+      <c r="D31" t="str">
         <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
       </c>
-      <c r="D31" t="str">
+      <c r="E31" t="str">
         <v>P2</v>
       </c>
-      <c r="E31" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F31" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G31" t="str">
+        <v>REQ-026, REQ-029</v>
+      </c>
+      <c r="H31" t="str">
         <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
       </c>
-      <c r="G31" t="str">
+      <c r="I31" t="str">
         <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
+        <v>REQ-031</v>
+      </c>
+      <c r="B32" t="str">
         <v>Infrastructure &amp; Déploiement</v>
       </c>
-      <c r="B32" t="str">
+      <c r="C32" t="str">
         <v>Versionning Git &amp; GitHub</v>
       </c>
-      <c r="C32" t="str">
+      <c r="D32" t="str">
         <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
       </c>
-      <c r="D32" t="str">
-        <v>P1</v>
-      </c>
       <c r="E32" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F32" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G32" t="str">
+        <v>REQ-005, REQ-029</v>
+      </c>
+      <c r="H32" t="str">
         <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
       </c>
-      <c r="G32" t="str">
+      <c r="I32" t="str">
         <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
+        <v>REQ-032</v>
+      </c>
+      <c r="B33" t="str">
         <v>Infrastructure &amp; Déploiement</v>
       </c>
-      <c r="B33" t="str">
+      <c r="C33" t="str">
         <v>API REST Fastify</v>
       </c>
-      <c r="C33" t="str">
+      <c r="D33" t="str">
         <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
       </c>
-      <c r="D33" t="str">
+      <c r="E33" t="str">
         <v>P0</v>
       </c>
-      <c r="E33" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F33" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G33" t="str">
+        <v>REQ-011, REQ-029</v>
+      </c>
+      <c r="H33" t="str">
         <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
       </c>
-      <c r="G33" t="str">
+      <c r="I33" t="str">
         <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
+        <v>REQ-033</v>
+      </c>
+      <c r="B34" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B34" t="str">
+      <c r="C34" t="str">
         <v>UI React + TypeScript + Vite</v>
       </c>
-      <c r="C34" t="str">
+      <c r="D34" t="str">
         <v>Bundling optimisé, HMR dev mode</v>
       </c>
-      <c r="D34" t="str">
-        <v>P1</v>
-      </c>
       <c r="E34" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F34" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G34" t="str">
+        <v>REQ-015, REQ-029</v>
+      </c>
+      <c r="H34" t="str">
         <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
       </c>
-      <c r="G34" t="str">
+      <c r="I34" t="str">
         <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
+        <v>REQ-034</v>
+      </c>
+      <c r="B35" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B35" t="str">
+      <c r="C35" t="str">
         <v>Configuration IA section</v>
       </c>
-      <c r="C35" t="str">
+      <c r="D35" t="str">
         <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
       </c>
-      <c r="D35" t="str">
-        <v>P1</v>
-      </c>
       <c r="E35" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F35" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G35" t="str">
+        <v>REQ-022, REQ-029</v>
+      </c>
+      <c r="H35" t="str">
         <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
       </c>
-      <c r="G35" t="str">
+      <c r="I35" t="str">
         <v>UX: clair et accessible, pas scroll nécessaire</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
+        <v>REQ-035</v>
+      </c>
+      <c r="B36" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B36" t="str">
+      <c r="C36" t="str">
         <v>Génération questions section</v>
       </c>
-      <c r="C36" t="str">
+      <c r="D36" t="str">
         <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
       </c>
-      <c r="D36" t="str">
-        <v>P1</v>
-      </c>
       <c r="E36" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F36" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G36" t="str">
+        <v>REQ-012, REQ-013, REQ-029</v>
+      </c>
+      <c r="H36" t="str">
         <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
       </c>
-      <c r="G36" t="str">
+      <c r="I36" t="str">
         <v>État uploadingReferential: loading indicator, disabled submit</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>REQ-036</v>
+      </c>
+      <c r="B37" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B37" t="str">
+      <c r="C37" t="str">
         <v>Référentiel documentaire section</v>
       </c>
-      <c r="C37" t="str">
+      <c r="D37" t="str">
         <v>Ajouter document avec métas, liste affichée</v>
       </c>
-      <c r="D37" t="str">
-        <v>P1</v>
-      </c>
       <c r="E37" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F37" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G37" t="str">
+        <v>REQ-017, REQ-018, REQ-029</v>
+      </c>
+      <c r="H37" t="str">
         <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
       </c>
-      <c r="G37" t="str">
+      <c r="I37" t="str">
         <v>Erreurs affichées, success feedback, état documentS refresh</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>REQ-037</v>
+      </c>
+      <c r="B38" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B38" t="str">
+      <c r="C38" t="str">
         <v>Échelles métriques config</v>
       </c>
-      <c r="C38" t="str">
+      <c r="D38" t="str">
         <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
       </c>
-      <c r="D38" t="str">
-        <v>P1</v>
-      </c>
       <c r="E38" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F38" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G38" t="str">
+        <v>REQ-019, REQ-020, REQ-029</v>
+      </c>
+      <c r="H38" t="str">
         <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
       </c>
-      <c r="G38" t="str">
+      <c r="I38" t="str">
         <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
+        <v>REQ-038</v>
+      </c>
+      <c r="B39" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B39" t="str">
+      <c r="C39" t="str">
         <v>Dashboard avec KPIs</v>
       </c>
-      <c r="C39" t="str">
+      <c r="D39" t="str">
         <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
       </c>
-      <c r="D39" t="str">
-        <v>P1</v>
-      </c>
       <c r="E39" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F39" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G39" t="str">
+        <v>-</v>
+      </c>
+      <c r="H39" t="str">
         <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
       </c>
-      <c r="G39" t="str">
+      <c r="I39" t="str">
         <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
+        <v>REQ-039</v>
+      </c>
+      <c r="B40" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B40" t="str">
+      <c r="C40" t="str">
         <v>Gestion entretiens</v>
       </c>
-      <c r="C40" t="str">
+      <c r="D40" t="str">
         <v>Interviewés, notes questions, scoring intégré</v>
       </c>
-      <c r="D40" t="str">
-        <v>P1</v>
-      </c>
       <c r="E40" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F40" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G40" t="str">
+        <v>-</v>
+      </c>
+      <c r="H40" t="str">
         <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
       </c>
-      <c r="G40" t="str">
+      <c r="I40" t="str">
         <v>Chaque note liée criterion + interviewee + score optionnel</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
+        <v>REQ-040</v>
+      </c>
+      <c r="B41" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B41" t="str">
+      <c r="C41" t="str">
         <v>Audit log viewer</v>
       </c>
-      <c r="C41" t="str">
+      <c r="D41" t="str">
         <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
       </c>
-      <c r="D41" t="str">
-        <v>P1</v>
-      </c>
       <c r="E41" t="str">
-        <v>Complété</v>
+        <v>P1</v>
       </c>
       <c r="F41" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G41" t="str">
+        <v>REQ-039</v>
+      </c>
+      <c r="H41" t="str">
         <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
       </c>
-      <c r="G41" t="str">
+      <c r="I41" t="str">
         <v>Sync knownActions dynamiquement depuis logs récupérés</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
+        <v>REQ-041</v>
+      </c>
+      <c r="B42" t="str">
         <v>UI/UX</v>
       </c>
-      <c r="B42" t="str">
+      <c r="C42" t="str">
         <v>Export buttons</v>
       </c>
-      <c r="C42" t="str">
+      <c r="D42" t="str">
         <v>Boutons DOCX et CSV téléchargement</v>
       </c>
-      <c r="D42" t="str">
+      <c r="E42" t="str">
         <v>P2</v>
       </c>
-      <c r="E42" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F42" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G42" t="str">
+        <v>-</v>
+      </c>
+      <c r="H42" t="str">
         <v>POST /export-report et /export-csv. browser Blob download.</v>
       </c>
-      <c r="G42" t="str">
+      <c r="I42" t="str">
         <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
+        <v>REQ-042</v>
+      </c>
+      <c r="B43" t="str">
         <v>Persévérance &amp; Facilité</v>
       </c>
-      <c r="B43" t="str">
+      <c r="C43" t="str">
         <v>Documentation complète</v>
       </c>
-      <c r="C43" t="str">
+      <c r="D43" t="str">
         <v>Setup guides, quickstart, git manual, examples références</v>
       </c>
-      <c r="D43" t="str">
+      <c r="E43" t="str">
         <v>P2</v>
       </c>
-      <c r="E43" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F43" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G43" t="str">
+        <v>-</v>
+      </c>
+      <c r="H43" t="str">
         <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
       </c>
-      <c r="G43" t="str">
+      <c r="I43" t="str">
         <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
       <c r="A44" t="str">
+        <v>REQ-043</v>
+      </c>
+      <c r="B44" t="str">
         <v>Persévérance &amp; Facilité</v>
       </c>
-      <c r="B44" t="str">
+      <c r="C44" t="str">
         <v>One-command installation</v>
       </c>
-      <c r="C44" t="str">
+      <c r="D44" t="str">
         <v>Non-tech user peut installer Rubis complet en 1 commande</v>
       </c>
-      <c r="D44" t="str">
+      <c r="E44" t="str">
         <v>P2</v>
       </c>
-      <c r="E44" t="str">
-        <v>Complété</v>
-      </c>
-      <c r="F44" t="str" xml:space="preserve">
+      <c r="F44" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G44" t="str">
+        <v>-</v>
+      </c>
+      <c r="H44" t="str" xml:space="preserve">
         <v xml:space="preserve">.
  install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
       </c>
-      <c r="G44" t="str">
+      <c r="I44" t="str">
         <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
       <c r="A45" t="str">
+        <v>REQ-044</v>
+      </c>
+      <c r="B45" t="str">
         <v>Persévérance &amp; Facilité</v>
       </c>
-      <c r="B45" t="str">
+      <c r="C45" t="str">
         <v>One-command launch</v>
       </c>
-      <c r="C45" t="str" xml:space="preserve">
+      <c r="D45" t="str" xml:space="preserve">
         <v xml:space="preserve">npm run dev ou .
 start-rubis.ps1 pour lancer tout</v>
       </c>
-      <c r="D45" t="str">
+      <c r="E45" t="str">
         <v>P2</v>
       </c>
-      <c r="E45" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F45" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G45" t="str">
+        <v>-</v>
+      </c>
+      <c r="H45" t="str">
         <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
       </c>
-      <c r="G45" t="str">
+      <c r="I45" t="str">
         <v>Détection auto erreurs, log output lisible</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
+        <v>REQ-045</v>
+      </c>
+      <c r="B46" t="str">
         <v>Persévérance &amp; Facilité</v>
       </c>
-      <c r="B46" t="str">
+      <c r="C46" t="str">
         <v>Clear error messages</v>
       </c>
-      <c r="C46" t="str">
+      <c r="D46" t="str">
         <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
       </c>
-      <c r="D46" t="str">
+      <c r="E46" t="str">
         <v>P2</v>
       </c>
-      <c r="E46" t="str">
-        <v>Complété</v>
-      </c>
       <c r="F46" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G46" t="str">
+        <v>-</v>
+      </c>
+      <c r="H46" t="str">
         <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
       </c>
-      <c r="G46" t="str">
+      <c r="I46" t="str">
         <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
+        <v>REQ-046</v>
+      </c>
+      <c r="B47" t="str">
         <v>Persévérance &amp; Facilité</v>
       </c>
-      <c r="B47" t="str">
+      <c r="C47" t="str">
         <v>Roadmap versioning</v>
       </c>
-      <c r="C47" t="str">
+      <c r="D47" t="str">
         <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
       </c>
-      <c r="D47" t="str">
+      <c r="E47" t="str">
         <v>P2</v>
       </c>
-      <c r="E47" t="str">
+      <c r="F47" t="str">
         <v>Planifié</v>
       </c>
-      <c r="F47" t="str">
+      <c r="G47" t="str">
+        <v>-</v>
+      </c>
+      <c r="H47" t="str">
         <v>Créer ROADMAP.xlsx avec specs, priorités, statuts, directives implémentation.</v>
       </c>
-      <c r="G47" t="str">
+      <c r="I47" t="str">
         <v>À committé dans git, mis à jour post-MVP pour v2 features</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Update roadmap with referential dropdown feature (REQ-003)
- Added new specification: Liste déroulante référentiels sécurité
- 47 specifications total (was 46)
- Updated dependency matrix (REQ-003 depends on REQ-002)
- All subsequent IDs shifted by 1
- ROADMAP.xlsx regenerated with new entry
</commit_message>
<xml_diff>
--- a/ROADMAP.xlsx
+++ b/ROADMAP.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I48"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -502,16 +502,16 @@
         <v>REQ-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Cœur métier</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C4" t="str">
-        <v>Gestion des critères d'audit</v>
+        <v>Liste déroulante référentiels sécurité</v>
       </c>
       <c r="D4" t="str">
-        <v>Code, titre, thème pour chaque critère avec lien campagne</v>
+        <v>Select avec 25+ référentiels organisés par catégories (ISO, France, Luxembourg, EU, International)</v>
       </c>
       <c r="E4" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F4" t="str">
         <v>Complété</v>
@@ -520,10 +520,10 @@
         <v>REQ-002</v>
       </c>
       <c r="H4" t="str">
-        <v>POST /criteria, GET /criteria?campaignId=. Clé étrangère campaignId.</v>
+        <v>Select dropdown dans form création campagne. Optgroups: ISO27001/27002/27005/19011, PASSI/LPM/II901/ANSSI/HDS/RGS, CSSF, NIS2/GDPR/DORA, NIST/CIS/SOC2/PCI-DSS/COBIT, Custom</v>
       </c>
       <c r="I4" t="str">
-        <v>Critères liés à campagnes pour isolation des données</v>
+        <v>Remplace input texte libre. Améliore UX et standardise les noms de référentiels. ~$*.xlsx ajouté au .gitignore</v>
       </c>
     </row>
     <row r="5">
@@ -534,10 +534,10 @@
         <v>Cœur métier</v>
       </c>
       <c r="C5" t="str">
-        <v>Génération de questions</v>
+        <v>Gestion des critères d'audit</v>
       </c>
       <c r="D5" t="str">
-        <v>Questions avec text, guidance, theme générées dynamiquement</v>
+        <v>Code, titre, thème pour chaque critère avec lien campagne</v>
       </c>
       <c r="E5" t="str">
         <v>P0</v>
@@ -546,13 +546,13 @@
         <v>Complété</v>
       </c>
       <c r="G5" t="str">
-        <v>REQ-003</v>
+        <v>REQ-002</v>
       </c>
       <c r="H5" t="str">
-        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
+        <v>POST /criteria, GET /criteria?campaignId=. Clé étrangère campaignId.</v>
       </c>
       <c r="I5" t="str">
-        <v>Peut être depuis template ou IA (voir section IA)</v>
+        <v>Critères liés à campagnes pour isolation des données</v>
       </c>
     </row>
     <row r="6">
@@ -560,28 +560,28 @@
         <v>REQ-005</v>
       </c>
       <c r="B6" t="str">
-        <v>IA &amp; Génération</v>
+        <v>Cœur métier</v>
       </c>
       <c r="C6" t="str">
-        <v>Génération depuis référentiel</v>
+        <v>Génération de questions</v>
       </c>
       <c r="D6" t="str">
-        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
+        <v>Questions avec text, guidance, theme générées dynamiquement</v>
       </c>
       <c r="E6" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F6" t="str">
         <v>Complété</v>
       </c>
       <c r="G6" t="str">
-        <v>REQ-003</v>
+        <v>REQ-004</v>
       </c>
       <c r="H6" t="str">
-        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
+        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
       </c>
       <c r="I6" t="str">
-        <v>Limite 50KB texte extrait pour perf API</v>
+        <v>Peut être depuis template ou IA (voir section IA)</v>
       </c>
     </row>
     <row r="7">
@@ -592,10 +592,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C7" t="str">
-        <v>Dual AI strategy - OpenAI</v>
+        <v>Génération depuis référentiel</v>
       </c>
       <c r="D7" t="str">
-        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
+        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
       </c>
       <c r="E7" t="str">
         <v>P1</v>
@@ -604,13 +604,13 @@
         <v>Complété</v>
       </c>
       <c r="G7" t="str">
-        <v>REQ-028</v>
+        <v>REQ-004</v>
       </c>
       <c r="H7" t="str">
-        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
+        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
       </c>
       <c r="I7" t="str">
-        <v>Fallback si OPENAI_API_KEY absent</v>
+        <v>Limite 50KB texte extrait pour perf API</v>
       </c>
     </row>
     <row r="8">
@@ -621,10 +621,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C8" t="str">
-        <v>Dual AI strategy - Ollama local</v>
+        <v>Dual AI strategy - OpenAI</v>
       </c>
       <c r="D8" t="str">
-        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
+        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
       </c>
       <c r="E8" t="str">
         <v>P1</v>
@@ -633,13 +633,13 @@
         <v>Complété</v>
       </c>
       <c r="G8" t="str">
-        <v>REQ-028</v>
+        <v>REQ-029</v>
       </c>
       <c r="H8" t="str">
-        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
+        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
       </c>
       <c r="I8" t="str">
-        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
+        <v>Fallback si OPENAI_API_KEY absent</v>
       </c>
     </row>
     <row r="9">
@@ -650,10 +650,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C9" t="str">
-        <v>Model switching UI</v>
+        <v>Dual AI strategy - Ollama local</v>
       </c>
       <c r="D9" t="str">
-        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
+        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
       </c>
       <c r="E9" t="str">
         <v>P1</v>
@@ -662,13 +662,13 @@
         <v>Complété</v>
       </c>
       <c r="G9" t="str">
-        <v>REQ-006, REQ-007</v>
+        <v>REQ-029</v>
       </c>
       <c r="H9" t="str">
-        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
+        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
       </c>
       <c r="I9" t="str">
-        <v>Changement runtime, pas besoin restart API</v>
+        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
       </c>
     </row>
     <row r="10">
@@ -679,10 +679,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C10" t="str">
-        <v>Parsing référentiel multi-format</v>
+        <v>Model switching UI</v>
       </c>
       <c r="D10" t="str">
-        <v>Support PDF et Excel avec extraction de texte</v>
+        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
       </c>
       <c r="E10" t="str">
         <v>P1</v>
@@ -691,13 +691,13 @@
         <v>Complété</v>
       </c>
       <c r="G10" t="str">
-        <v>REQ-005</v>
+        <v>REQ-007, REQ-008</v>
       </c>
       <c r="H10" t="str">
-        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
+        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
       </c>
       <c r="I10" t="str">
-        <v>Gère encodages UTF-8, caractères spéciaux</v>
+        <v>Changement runtime, pas besoin restart API</v>
       </c>
     </row>
     <row r="11">
@@ -708,10 +708,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C11" t="str">
-        <v>Prompt dynamique contextuel</v>
+        <v>Parsing référentiel multi-format</v>
       </c>
       <c r="D11" t="str">
-        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
+        <v>Support PDF et Excel avec extraction de texte</v>
       </c>
       <c r="E11" t="str">
         <v>P1</v>
@@ -720,13 +720,13 @@
         <v>Complété</v>
       </c>
       <c r="G11" t="str">
-        <v>REQ-005</v>
+        <v>REQ-006</v>
       </c>
       <c r="H11" t="str">
-        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
+        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
       </c>
       <c r="I11" t="str">
-        <v>Zod validation sur count (1-10), language (fr/en)</v>
+        <v>Gère encodages UTF-8, caractères spéciaux</v>
       </c>
     </row>
     <row r="12">
@@ -734,28 +734,28 @@
         <v>REQ-011</v>
       </c>
       <c r="B12" t="str">
-        <v>Structuration données</v>
+        <v>IA &amp; Génération</v>
       </c>
       <c r="C12" t="str">
-        <v>Modèle Document</v>
+        <v>Prompt dynamique contextuel</v>
       </c>
       <c r="D12" t="str">
-        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
+        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
       </c>
       <c r="E12" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F12" t="str">
         <v>Complété</v>
       </c>
       <c r="G12" t="str">
-        <v>REQ-002</v>
+        <v>REQ-006</v>
       </c>
       <c r="H12" t="str">
-        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
+        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
       </c>
       <c r="I12" t="str">
-        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
+        <v>Zod validation sur count (1-10), language (fr/en)</v>
       </c>
     </row>
     <row r="13">
@@ -766,10 +766,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C13" t="str">
-        <v>Modèle Interviewé</v>
+        <v>Modèle Document</v>
       </c>
       <c r="D13" t="str">
-        <v>Nom complet, rôle, lié à campaign</v>
+        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
       </c>
       <c r="E13" t="str">
         <v>P0</v>
@@ -781,10 +781,10 @@
         <v>REQ-002</v>
       </c>
       <c r="H13" t="str">
-        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
+        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
       </c>
       <c r="I13" t="str">
-        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
+        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
       </c>
     </row>
     <row r="14">
@@ -795,10 +795,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C14" t="str">
-        <v>Modèle Note d'entretien</v>
+        <v>Modèle Interviewé</v>
       </c>
       <c r="D14" t="str">
-        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
+        <v>Nom complet, rôle, lié à campaign</v>
       </c>
       <c r="E14" t="str">
         <v>P0</v>
@@ -807,13 +807,13 @@
         <v>Complété</v>
       </c>
       <c r="G14" t="str">
-        <v>REQ-003, REQ-012</v>
+        <v>REQ-002</v>
       </c>
       <c r="H14" t="str">
-        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
+        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
       </c>
       <c r="I14" t="str">
-        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
+        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
       </c>
     </row>
     <row r="15">
@@ -824,25 +824,25 @@
         <v>Structuration données</v>
       </c>
       <c r="C15" t="str">
-        <v>Matrice de conformité</v>
+        <v>Modèle Note d'entretien</v>
       </c>
       <c r="D15" t="str">
-        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
+        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
       </c>
       <c r="E15" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F15" t="str">
         <v>Complété</v>
       </c>
       <c r="G15" t="str">
-        <v>REQ-013</v>
+        <v>REQ-004, REQ-013</v>
       </c>
       <c r="H15" t="str">
-        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
+        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
       </c>
       <c r="I15" t="str">
-        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
+        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
       </c>
     </row>
     <row r="16">
@@ -853,10 +853,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C16" t="str">
-        <v>Configuration Métriques</v>
+        <v>Matrice de conformité</v>
       </c>
       <c r="D16" t="str">
-        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
+        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
       </c>
       <c r="E16" t="str">
         <v>P1</v>
@@ -865,13 +865,13 @@
         <v>Complété</v>
       </c>
       <c r="G16" t="str">
-        <v>REQ-002</v>
+        <v>REQ-014</v>
       </c>
       <c r="H16" t="str">
-        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
+        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
       </c>
       <c r="I16" t="str">
-        <v>Format texte (ex: '1-5') pour flexibilité</v>
+        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
       </c>
     </row>
     <row r="17">
@@ -879,13 +879,13 @@
         <v>REQ-016</v>
       </c>
       <c r="B17" t="str">
-        <v>Audit &amp; Traçabilité</v>
+        <v>Structuration données</v>
       </c>
       <c r="C17" t="str">
-        <v>Audit Log complet</v>
+        <v>Configuration Métriques</v>
       </c>
       <c r="D17" t="str">
-        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
+        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
       </c>
       <c r="E17" t="str">
         <v>P1</v>
@@ -894,13 +894,13 @@
         <v>Complété</v>
       </c>
       <c r="G17" t="str">
-        <v>REQ-002, REQ-028</v>
+        <v>REQ-002</v>
       </c>
       <c r="H17" t="str">
-        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
+        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
       </c>
       <c r="I17" t="str">
-        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
+        <v>Format texte (ex: '1-5') pour flexibilité</v>
       </c>
     </row>
     <row r="18">
@@ -911,10 +911,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C18" t="str">
-        <v>Filtrage logs par période</v>
+        <v>Audit Log complet</v>
       </c>
       <c r="D18" t="str">
-        <v>Vue 7j, 30j, tout (by date range filter)</v>
+        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
       </c>
       <c r="E18" t="str">
         <v>P1</v>
@@ -923,13 +923,13 @@
         <v>Complété</v>
       </c>
       <c r="G18" t="str">
-        <v>REQ-016</v>
+        <v>REQ-002, REQ-029</v>
       </c>
       <c r="H18" t="str">
-        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
+        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
       </c>
       <c r="I18" t="str">
-        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
+        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
       </c>
     </row>
     <row r="19">
@@ -940,10 +940,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C19" t="str">
-        <v>Filtrage logs par action</v>
+        <v>Filtrage logs par période</v>
       </c>
       <c r="D19" t="str">
-        <v>Filter sur type d'action (campaign.created, etc.)</v>
+        <v>Vue 7j, 30j, tout (by date range filter)</v>
       </c>
       <c r="E19" t="str">
         <v>P1</v>
@@ -952,13 +952,13 @@
         <v>Complété</v>
       </c>
       <c r="G19" t="str">
-        <v>REQ-016</v>
+        <v>REQ-017</v>
       </c>
       <c r="H19" t="str">
-        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
+        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
       </c>
       <c r="I19" t="str">
-        <v>Enum actions découvertes dynamiquement from logs</v>
+        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
       </c>
     </row>
     <row r="20">
@@ -966,28 +966,28 @@
         <v>REQ-019</v>
       </c>
       <c r="B20" t="str">
-        <v>Rapports &amp; Exports</v>
+        <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C20" t="str">
-        <v>Export DOCX</v>
+        <v>Filtrage logs par action</v>
       </c>
       <c r="D20" t="str">
-        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
+        <v>Filter sur type d'action (campaign.created, etc.)</v>
       </c>
       <c r="E20" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F20" t="str">
         <v>Complété</v>
       </c>
       <c r="G20" t="str">
-        <v>REQ-004, REQ-014</v>
+        <v>REQ-017</v>
       </c>
       <c r="H20" t="str">
-        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
+        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
       </c>
       <c r="I20" t="str">
-        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
+        <v>Enum actions découvertes dynamiquement from logs</v>
       </c>
     </row>
     <row r="21">
@@ -998,10 +998,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C21" t="str">
-        <v>Export CSV</v>
+        <v>Export DOCX</v>
       </c>
       <c r="D21" t="str">
-        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
+        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
       </c>
       <c r="E21" t="str">
         <v>P2</v>
@@ -1010,13 +1010,13 @@
         <v>Complété</v>
       </c>
       <c r="G21" t="str">
-        <v>REQ-014, REQ-016</v>
+        <v>REQ-005, REQ-015</v>
       </c>
       <c r="H21" t="str">
-        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
+        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
       </c>
       <c r="I21" t="str">
-        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
+        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
       </c>
     </row>
     <row r="22">
@@ -1027,10 +1027,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C22" t="str">
-        <v>Gestion des rapports</v>
+        <v>Export CSV</v>
       </c>
       <c r="D22" t="str">
-        <v>Stocker rapports générés avec titre, date gen, version</v>
+        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
       </c>
       <c r="E22" t="str">
         <v>P2</v>
@@ -1039,13 +1039,13 @@
         <v>Complété</v>
       </c>
       <c r="G22" t="str">
-        <v>REQ-019, REQ-020</v>
+        <v>REQ-015, REQ-017</v>
       </c>
       <c r="H22" t="str">
-        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
+        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
       </c>
       <c r="I22" t="str">
-        <v>Récupérable dans UI, archivé pour traçabilité</v>
+        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
       </c>
     </row>
     <row r="23">
@@ -1053,28 +1053,28 @@
         <v>REQ-022</v>
       </c>
       <c r="B23" t="str">
-        <v>Dashboard &amp; Visualisation</v>
+        <v>Rapports &amp; Exports</v>
       </c>
       <c r="C23" t="str">
-        <v>KPIs essentiels</v>
+        <v>Gestion des rapports</v>
       </c>
       <c r="D23" t="str">
-        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
+        <v>Stocker rapports générés avec titre, date gen, version</v>
       </c>
       <c r="E23" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F23" t="str">
         <v>Complété</v>
       </c>
       <c r="G23" t="str">
-        <v>REQ-011, REQ-012, REQ-013</v>
+        <v>REQ-020, REQ-021</v>
       </c>
       <c r="H23" t="str">
-        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
+        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
       </c>
       <c r="I23" t="str">
-        <v>Affiché en gros chiffres zone haute dashboard</v>
+        <v>Récupérable dans UI, archivé pour traçabilité</v>
       </c>
     </row>
     <row r="24">
@@ -1085,25 +1085,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C24" t="str">
-        <v>Matrice de conformité interactive</v>
+        <v>KPIs essentiels</v>
       </c>
       <c r="D24" t="str">
-        <v>Tableau avec % conformité par criterion, tri/filtre</v>
+        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
       </c>
       <c r="E24" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F24" t="str">
         <v>Complété</v>
       </c>
       <c r="G24" t="str">
-        <v>REQ-014</v>
+        <v>REQ-012, REQ-013, REQ-014</v>
       </c>
       <c r="H24" t="str">
-        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
+        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
       </c>
       <c r="I24" t="str">
-        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
+        <v>Affiché en gros chiffres zone haute dashboard</v>
       </c>
     </row>
     <row r="25">
@@ -1114,25 +1114,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C25" t="str">
-        <v>Graphiques optionnels (futur)</v>
+        <v>Matrice de conformité interactive</v>
       </c>
       <c r="D25" t="str">
-        <v>Tendances audit timeline, pie charts conformity domains</v>
+        <v>Tableau avec % conformité par criterion, tri/filtre</v>
       </c>
       <c r="E25" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="F25" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G25" t="str">
-        <v>REQ-022</v>
+        <v>REQ-015</v>
       </c>
       <c r="H25" t="str">
-        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
+        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
       </c>
       <c r="I25" t="str">
-        <v>MVP n'a pas graphiques, architecture prête pour.</v>
+        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
       </c>
     </row>
     <row r="26">
@@ -1140,28 +1140,28 @@
         <v>REQ-025</v>
       </c>
       <c r="B26" t="str">
-        <v>Configuration &amp; Flexibilité</v>
+        <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C26" t="str">
-        <v>Support multilingue</v>
+        <v>Graphiques optionnels (futur)</v>
       </c>
       <c r="D26" t="str">
-        <v>FR et EN, sélection par campaign</v>
+        <v>Tendances audit timeline, pie charts conformity domains</v>
       </c>
       <c r="E26" t="str">
-        <v>P1</v>
+        <v>P3</v>
       </c>
       <c r="F26" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G26" t="str">
-        <v>REQ-028</v>
+        <v>REQ-023</v>
       </c>
       <c r="H26" t="str">
-        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
+        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
       </c>
       <c r="I26" t="str">
-        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
+        <v>MVP n'a pas graphiques, architecture prête pour.</v>
       </c>
     </row>
     <row r="27">
@@ -1172,10 +1172,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C27" t="str">
-        <v>Modèle Ollama configurable</v>
+        <v>Support multilingue</v>
       </c>
       <c r="D27" t="str">
-        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
+        <v>FR et EN, sélection par campaign</v>
       </c>
       <c r="E27" t="str">
         <v>P1</v>
@@ -1184,13 +1184,13 @@
         <v>Complété</v>
       </c>
       <c r="G27" t="str">
-        <v>REQ-007</v>
+        <v>REQ-029</v>
       </c>
       <c r="H27" t="str">
-        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
+        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
       </c>
       <c r="I27" t="str">
-        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
+        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
       </c>
     </row>
     <row r="28">
@@ -1201,10 +1201,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C28" t="str">
-        <v>OpenAI optionnel</v>
+        <v>Modèle Ollama configurable</v>
       </c>
       <c r="D28" t="str">
-        <v>API key via .env, fallback auto Ollama si absent</v>
+        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
       </c>
       <c r="E28" t="str">
         <v>P1</v>
@@ -1213,13 +1213,13 @@
         <v>Complété</v>
       </c>
       <c r="G28" t="str">
-        <v>REQ-028</v>
+        <v>REQ-008</v>
       </c>
       <c r="H28" t="str">
-        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
+        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
       </c>
       <c r="I28" t="str">
-        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
+        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
       </c>
     </row>
     <row r="29">
@@ -1230,25 +1230,25 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C29" t="str">
-        <v>Thèmes personnalisés</v>
+        <v>OpenAI optionnel</v>
       </c>
       <c r="D29" t="str">
-        <v>Texte libre pour documents et questions</v>
+        <v>API key via .env, fallback auto Ollama si absent</v>
       </c>
       <c r="E29" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F29" t="str">
         <v>Complété</v>
       </c>
       <c r="G29" t="str">
-        <v>-</v>
+        <v>REQ-029</v>
       </c>
       <c r="H29" t="str">
-        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
+        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
       </c>
       <c r="I29" t="str">
-        <v>Permet flexibilité sur domaines audit custom</v>
+        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
       </c>
     </row>
     <row r="30">
@@ -1256,16 +1256,16 @@
         <v>REQ-029</v>
       </c>
       <c r="B30" t="str">
-        <v>Infrastructure &amp; Déploiement</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C30" t="str">
-        <v>Offline-first capability</v>
+        <v>Thèmes personnalisés</v>
       </c>
       <c r="D30" t="str">
-        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
+        <v>Texte libre pour documents et questions</v>
       </c>
       <c r="E30" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F30" t="str">
         <v>Complété</v>
@@ -1274,10 +1274,10 @@
         <v>-</v>
       </c>
       <c r="H30" t="str">
-        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
+        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
       </c>
       <c r="I30" t="str">
-        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
+        <v>Permet flexibilité sur domaines audit custom</v>
       </c>
     </row>
     <row r="31">
@@ -1288,25 +1288,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C31" t="str">
-        <v>Automation PowerShell</v>
+        <v>Offline-first capability</v>
       </c>
       <c r="D31" t="str">
-        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
+        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
       </c>
       <c r="E31" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F31" t="str">
         <v>Complété</v>
       </c>
       <c r="G31" t="str">
-        <v>REQ-026, REQ-029</v>
+        <v>-</v>
       </c>
       <c r="H31" t="str">
-        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
+        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
       </c>
       <c r="I31" t="str">
-        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
+        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
       </c>
     </row>
     <row r="32">
@@ -1317,25 +1317,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C32" t="str">
-        <v>Versionning Git &amp; GitHub</v>
+        <v>Automation PowerShell</v>
       </c>
       <c r="D32" t="str">
-        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
+        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
       </c>
       <c r="E32" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F32" t="str">
         <v>Complété</v>
       </c>
       <c r="G32" t="str">
-        <v>REQ-005, REQ-029</v>
+        <v>REQ-027, REQ-030</v>
       </c>
       <c r="H32" t="str">
-        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
+        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
       </c>
       <c r="I32" t="str">
-        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
+        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
       </c>
     </row>
     <row r="33">
@@ -1346,25 +1346,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C33" t="str">
-        <v>API REST Fastify</v>
+        <v>Versionning Git &amp; GitHub</v>
       </c>
       <c r="D33" t="str">
-        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
+        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
       </c>
       <c r="E33" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F33" t="str">
         <v>Complété</v>
       </c>
       <c r="G33" t="str">
-        <v>REQ-011, REQ-029</v>
+        <v>REQ-006, REQ-030</v>
       </c>
       <c r="H33" t="str">
-        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
+        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
       </c>
       <c r="I33" t="str">
-        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
+        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
       </c>
     </row>
     <row r="34">
@@ -1372,28 +1372,28 @@
         <v>REQ-033</v>
       </c>
       <c r="B34" t="str">
-        <v>UI/UX</v>
+        <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C34" t="str">
-        <v>UI React + TypeScript + Vite</v>
+        <v>API REST Fastify</v>
       </c>
       <c r="D34" t="str">
-        <v>Bundling optimisé, HMR dev mode</v>
+        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
       </c>
       <c r="E34" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F34" t="str">
         <v>Complété</v>
       </c>
       <c r="G34" t="str">
-        <v>REQ-015, REQ-029</v>
+        <v>REQ-012, REQ-030</v>
       </c>
       <c r="H34" t="str">
-        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
+        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
       </c>
       <c r="I34" t="str">
-        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
+        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
       </c>
     </row>
     <row r="35">
@@ -1404,10 +1404,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C35" t="str">
-        <v>Configuration IA section</v>
+        <v>UI React + TypeScript + Vite</v>
       </c>
       <c r="D35" t="str">
-        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
+        <v>Bundling optimisé, HMR dev mode</v>
       </c>
       <c r="E35" t="str">
         <v>P1</v>
@@ -1416,13 +1416,13 @@
         <v>Complété</v>
       </c>
       <c r="G35" t="str">
-        <v>REQ-022, REQ-029</v>
+        <v>REQ-016, REQ-030</v>
       </c>
       <c r="H35" t="str">
-        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
+        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
       </c>
       <c r="I35" t="str">
-        <v>UX: clair et accessible, pas scroll nécessaire</v>
+        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
       </c>
     </row>
     <row r="36">
@@ -1433,10 +1433,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C36" t="str">
-        <v>Génération questions section</v>
+        <v>Configuration IA section</v>
       </c>
       <c r="D36" t="str">
-        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
+        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
       </c>
       <c r="E36" t="str">
         <v>P1</v>
@@ -1445,13 +1445,13 @@
         <v>Complété</v>
       </c>
       <c r="G36" t="str">
-        <v>REQ-012, REQ-013, REQ-029</v>
+        <v>REQ-023, REQ-030</v>
       </c>
       <c r="H36" t="str">
-        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
+        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
       </c>
       <c r="I36" t="str">
-        <v>État uploadingReferential: loading indicator, disabled submit</v>
+        <v>UX: clair et accessible, pas scroll nécessaire</v>
       </c>
     </row>
     <row r="37">
@@ -1462,10 +1462,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C37" t="str">
-        <v>Référentiel documentaire section</v>
+        <v>Génération questions section</v>
       </c>
       <c r="D37" t="str">
-        <v>Ajouter document avec métas, liste affichée</v>
+        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
       </c>
       <c r="E37" t="str">
         <v>P1</v>
@@ -1474,13 +1474,13 @@
         <v>Complété</v>
       </c>
       <c r="G37" t="str">
-        <v>REQ-017, REQ-018, REQ-029</v>
+        <v>REQ-013, REQ-014, REQ-030</v>
       </c>
       <c r="H37" t="str">
-        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
+        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
       </c>
       <c r="I37" t="str">
-        <v>Erreurs affichées, success feedback, état documentS refresh</v>
+        <v>État uploadingReferential: loading indicator, disabled submit</v>
       </c>
     </row>
     <row r="38">
@@ -1491,10 +1491,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C38" t="str">
-        <v>Échelles métriques config</v>
+        <v>Référentiel documentaire section</v>
       </c>
       <c r="D38" t="str">
-        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
+        <v>Ajouter document avec métas, liste affichée</v>
       </c>
       <c r="E38" t="str">
         <v>P1</v>
@@ -1503,13 +1503,13 @@
         <v>Complété</v>
       </c>
       <c r="G38" t="str">
-        <v>REQ-019, REQ-020, REQ-029</v>
+        <v>REQ-018, REQ-019, REQ-030</v>
       </c>
       <c r="H38" t="str">
-        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
+        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
       </c>
       <c r="I38" t="str">
-        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
+        <v>Erreurs affichées, success feedback, état documentS refresh</v>
       </c>
     </row>
     <row r="39">
@@ -1520,10 +1520,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C39" t="str">
-        <v>Dashboard avec KPIs</v>
+        <v>Échelles métriques config</v>
       </c>
       <c r="D39" t="str">
-        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
+        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
       </c>
       <c r="E39" t="str">
         <v>P1</v>
@@ -1532,13 +1532,13 @@
         <v>Complété</v>
       </c>
       <c r="G39" t="str">
-        <v>-</v>
+        <v>REQ-020, REQ-021, REQ-030</v>
       </c>
       <c r="H39" t="str">
-        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
+        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
       </c>
       <c r="I39" t="str">
-        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
+        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
       </c>
     </row>
     <row r="40">
@@ -1549,10 +1549,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C40" t="str">
-        <v>Gestion entretiens</v>
+        <v>Dashboard avec KPIs</v>
       </c>
       <c r="D40" t="str">
-        <v>Interviewés, notes questions, scoring intégré</v>
+        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
       </c>
       <c r="E40" t="str">
         <v>P1</v>
@@ -1564,10 +1564,10 @@
         <v>-</v>
       </c>
       <c r="H40" t="str">
-        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
+        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
       </c>
       <c r="I40" t="str">
-        <v>Chaque note liée criterion + interviewee + score optionnel</v>
+        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
       </c>
     </row>
     <row r="41">
@@ -1578,10 +1578,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C41" t="str">
-        <v>Audit log viewer</v>
+        <v>Gestion entretiens</v>
       </c>
       <c r="D41" t="str">
-        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
+        <v>Interviewés, notes questions, scoring intégré</v>
       </c>
       <c r="E41" t="str">
         <v>P1</v>
@@ -1590,13 +1590,13 @@
         <v>Complété</v>
       </c>
       <c r="G41" t="str">
-        <v>REQ-039</v>
+        <v>-</v>
       </c>
       <c r="H41" t="str">
-        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
+        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
       </c>
       <c r="I41" t="str">
-        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
+        <v>Chaque note liée criterion + interviewee + score optionnel</v>
       </c>
     </row>
     <row r="42">
@@ -1607,25 +1607,25 @@
         <v>UI/UX</v>
       </c>
       <c r="C42" t="str">
-        <v>Export buttons</v>
+        <v>Audit log viewer</v>
       </c>
       <c r="D42" t="str">
-        <v>Boutons DOCX et CSV téléchargement</v>
+        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
       </c>
       <c r="E42" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F42" t="str">
         <v>Complété</v>
       </c>
       <c r="G42" t="str">
-        <v>-</v>
+        <v>REQ-040</v>
       </c>
       <c r="H42" t="str">
-        <v>POST /export-report et /export-csv. browser Blob download.</v>
+        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
       </c>
       <c r="I42" t="str">
-        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
       </c>
     </row>
     <row r="43">
@@ -1633,13 +1633,13 @@
         <v>REQ-042</v>
       </c>
       <c r="B43" t="str">
-        <v>Persévérance &amp; Facilité</v>
+        <v>UI/UX</v>
       </c>
       <c r="C43" t="str">
-        <v>Documentation complète</v>
+        <v>Export buttons</v>
       </c>
       <c r="D43" t="str">
-        <v>Setup guides, quickstart, git manual, examples références</v>
+        <v>Boutons DOCX et CSV téléchargement</v>
       </c>
       <c r="E43" t="str">
         <v>P2</v>
@@ -1651,13 +1651,13 @@
         <v>-</v>
       </c>
       <c r="H43" t="str">
-        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
+        <v>POST /export-report et /export-csv. browser Blob download.</v>
       </c>
       <c r="I43" t="str">
-        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
+        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+      </c>
+    </row>
+    <row r="44">
       <c r="A44" t="str">
         <v>REQ-043</v>
       </c>
@@ -1665,10 +1665,10 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C44" t="str">
-        <v>One-command installation</v>
+        <v>Documentation complète</v>
       </c>
       <c r="D44" t="str">
-        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+        <v>Setup guides, quickstart, git manual, examples références</v>
       </c>
       <c r="E44" t="str">
         <v>P2</v>
@@ -1679,12 +1679,11 @@
       <c r="G44" t="str">
         <v>-</v>
       </c>
-      <c r="H44" t="str" xml:space="preserve">
-        <v xml:space="preserve">.
- install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      <c r="H44" t="str">
+        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
       </c>
       <c r="I44" t="str">
-        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -1695,41 +1694,42 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C45" t="str">
+        <v>One-command installation</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+      </c>
+      <c r="E45" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G45" t="str">
+        <v>-</v>
+      </c>
+      <c r="H45" t="str" xml:space="preserve">
+        <v xml:space="preserve">.
+ install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      </c>
+      <c r="I45" t="str">
+        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
+        <v>REQ-045</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C46" t="str">
         <v>One-command launch</v>
       </c>
-      <c r="D45" t="str" xml:space="preserve">
+      <c r="D46" t="str" xml:space="preserve">
         <v xml:space="preserve">npm run dev ou .
 start-rubis.ps1 pour lancer tout</v>
       </c>
-      <c r="E45" t="str">
-        <v>P2</v>
-      </c>
-      <c r="F45" t="str">
-        <v>Complété</v>
-      </c>
-      <c r="G45" t="str">
-        <v>-</v>
-      </c>
-      <c r="H45" t="str">
-        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
-      </c>
-      <c r="I45" t="str">
-        <v>Détection auto erreurs, log output lisible</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>REQ-045</v>
-      </c>
-      <c r="B46" t="str">
-        <v>Persévérance &amp; Facilité</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Clear error messages</v>
-      </c>
-      <c r="D46" t="str">
-        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
-      </c>
       <c r="E46" t="str">
         <v>P2</v>
       </c>
@@ -1740,10 +1740,10 @@
         <v>-</v>
       </c>
       <c r="H46" t="str">
-        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
       </c>
       <c r="I46" t="str">
-        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+        <v>Détection auto erreurs, log output lisible</v>
       </c>
     </row>
     <row r="47">
@@ -1754,30 +1754,59 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C47" t="str">
-        <v>Roadmap versioning</v>
+        <v>Clear error messages</v>
       </c>
       <c r="D47" t="str">
-        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
       </c>
       <c r="E47" t="str">
         <v>P2</v>
       </c>
       <c r="F47" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G47" t="str">
         <v>-</v>
       </c>
       <c r="H47" t="str">
+        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>REQ-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Roadmap versioning</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+      </c>
+      <c r="E48" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Planifié</v>
+      </c>
+      <c r="G48" t="str">
+        <v>-</v>
+      </c>
+      <c r="H48" t="str">
         <v>Créer ROADMAP.xlsx avec specs, priorités, statuts, directives implémentation.</v>
       </c>
-      <c r="I47" t="str">
+      <c r="I48" t="str">
         <v>À committé dans git, mis à jour post-MVP pour v2 features</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I47"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Add admin module for referentials management to roadmap (REQ-004)
- New specification: Module administration des référentiels
- Domain: Configuration & Flexibilité
- Priority: P2
- Status: Planifié
- Features: CRUD endpoints, UI table éditable, import/export JSON
- Dependencies: REQ-003 (liste référentiels) + REQ-030 (API)
- Total: 48 specifications (was 47)
- All subsequent IDs shifted by +1
</commit_message>
<xml_diff>
--- a/ROADMAP.xlsx
+++ b/ROADMAP.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I49"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -531,28 +531,28 @@
         <v>REQ-004</v>
       </c>
       <c r="B5" t="str">
-        <v>Cœur métier</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C5" t="str">
-        <v>Gestion des critères d'audit</v>
+        <v>Module administration des référentiels</v>
       </c>
       <c r="D5" t="str">
-        <v>Code, titre, thème pour chaque critère avec lien campagne</v>
+        <v>Interface admin pour ajouter/modifier/supprimer les référentiels disponibles dynamiquement</v>
       </c>
       <c r="E5" t="str">
-        <v>P0</v>
+        <v>P2</v>
       </c>
       <c r="F5" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G5" t="str">
-        <v>REQ-002</v>
+        <v>REQ-003, REQ-030</v>
       </c>
       <c r="H5" t="str">
-        <v>POST /criteria, GET /criteria?campaignId=. Clé étrangère campaignId.</v>
+        <v>Section admin protégée. CRUD référentiels: POST/PUT/DELETE /admin/referentials. Stockage db.data.referentials avec {id, name, category, description, isActive}. UI table éditable avec formulaire modal.</v>
       </c>
       <c r="I5" t="str">
-        <v>Critères liés à campagnes pour isolation des données</v>
+        <v>Permet personnalisation sans modifier le code. Validation côté serveur. Export/Import JSON pour backup.</v>
       </c>
     </row>
     <row r="6">
@@ -563,10 +563,10 @@
         <v>Cœur métier</v>
       </c>
       <c r="C6" t="str">
-        <v>Génération de questions</v>
+        <v>Gestion des critères d'audit</v>
       </c>
       <c r="D6" t="str">
-        <v>Questions avec text, guidance, theme générées dynamiquement</v>
+        <v>Code, titre, thème pour chaque critère avec lien campagne</v>
       </c>
       <c r="E6" t="str">
         <v>P0</v>
@@ -575,13 +575,13 @@
         <v>Complété</v>
       </c>
       <c r="G6" t="str">
-        <v>REQ-004</v>
+        <v>REQ-002</v>
       </c>
       <c r="H6" t="str">
-        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
+        <v>POST /criteria, GET /criteria?campaignId=. Clé étrangère campaignId.</v>
       </c>
       <c r="I6" t="str">
-        <v>Peut être depuis template ou IA (voir section IA)</v>
+        <v>Critères liés à campagnes pour isolation des données</v>
       </c>
     </row>
     <row r="7">
@@ -589,28 +589,28 @@
         <v>REQ-006</v>
       </c>
       <c r="B7" t="str">
-        <v>IA &amp; Génération</v>
+        <v>Cœur métier</v>
       </c>
       <c r="C7" t="str">
-        <v>Génération depuis référentiel</v>
+        <v>Génération de questions</v>
       </c>
       <c r="D7" t="str">
-        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
+        <v>Questions avec text, guidance, theme générées dynamiquement</v>
       </c>
       <c r="E7" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F7" t="str">
         <v>Complété</v>
       </c>
       <c r="G7" t="str">
-        <v>REQ-004</v>
+        <v>REQ-005</v>
       </c>
       <c r="H7" t="str">
-        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
+        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
       </c>
       <c r="I7" t="str">
-        <v>Limite 50KB texte extrait pour perf API</v>
+        <v>Peut être depuis template ou IA (voir section IA)</v>
       </c>
     </row>
     <row r="8">
@@ -621,10 +621,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C8" t="str">
-        <v>Dual AI strategy - OpenAI</v>
+        <v>Génération depuis référentiel</v>
       </c>
       <c r="D8" t="str">
-        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
+        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
       </c>
       <c r="E8" t="str">
         <v>P1</v>
@@ -633,13 +633,13 @@
         <v>Complété</v>
       </c>
       <c r="G8" t="str">
-        <v>REQ-029</v>
+        <v>REQ-005</v>
       </c>
       <c r="H8" t="str">
-        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
+        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
       </c>
       <c r="I8" t="str">
-        <v>Fallback si OPENAI_API_KEY absent</v>
+        <v>Limite 50KB texte extrait pour perf API</v>
       </c>
     </row>
     <row r="9">
@@ -650,10 +650,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C9" t="str">
-        <v>Dual AI strategy - Ollama local</v>
+        <v>Dual AI strategy - OpenAI</v>
       </c>
       <c r="D9" t="str">
-        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
+        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
       </c>
       <c r="E9" t="str">
         <v>P1</v>
@@ -662,13 +662,13 @@
         <v>Complété</v>
       </c>
       <c r="G9" t="str">
-        <v>REQ-029</v>
+        <v>REQ-030</v>
       </c>
       <c r="H9" t="str">
-        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
+        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
       </c>
       <c r="I9" t="str">
-        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
+        <v>Fallback si OPENAI_API_KEY absent</v>
       </c>
     </row>
     <row r="10">
@@ -679,10 +679,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C10" t="str">
-        <v>Model switching UI</v>
+        <v>Dual AI strategy - Ollama local</v>
       </c>
       <c r="D10" t="str">
-        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
+        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
       </c>
       <c r="E10" t="str">
         <v>P1</v>
@@ -691,13 +691,13 @@
         <v>Complété</v>
       </c>
       <c r="G10" t="str">
-        <v>REQ-007, REQ-008</v>
+        <v>REQ-030</v>
       </c>
       <c r="H10" t="str">
-        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
+        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
       </c>
       <c r="I10" t="str">
-        <v>Changement runtime, pas besoin restart API</v>
+        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
       </c>
     </row>
     <row r="11">
@@ -708,10 +708,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C11" t="str">
-        <v>Parsing référentiel multi-format</v>
+        <v>Model switching UI</v>
       </c>
       <c r="D11" t="str">
-        <v>Support PDF et Excel avec extraction de texte</v>
+        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
       </c>
       <c r="E11" t="str">
         <v>P1</v>
@@ -720,13 +720,13 @@
         <v>Complété</v>
       </c>
       <c r="G11" t="str">
-        <v>REQ-006</v>
+        <v>REQ-008, REQ-009</v>
       </c>
       <c r="H11" t="str">
-        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
+        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
       </c>
       <c r="I11" t="str">
-        <v>Gère encodages UTF-8, caractères spéciaux</v>
+        <v>Changement runtime, pas besoin restart API</v>
       </c>
     </row>
     <row r="12">
@@ -737,10 +737,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C12" t="str">
-        <v>Prompt dynamique contextuel</v>
+        <v>Parsing référentiel multi-format</v>
       </c>
       <c r="D12" t="str">
-        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
+        <v>Support PDF et Excel avec extraction de texte</v>
       </c>
       <c r="E12" t="str">
         <v>P1</v>
@@ -749,13 +749,13 @@
         <v>Complété</v>
       </c>
       <c r="G12" t="str">
-        <v>REQ-006</v>
+        <v>REQ-007</v>
       </c>
       <c r="H12" t="str">
-        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
+        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
       </c>
       <c r="I12" t="str">
-        <v>Zod validation sur count (1-10), language (fr/en)</v>
+        <v>Gère encodages UTF-8, caractères spéciaux</v>
       </c>
     </row>
     <row r="13">
@@ -763,28 +763,28 @@
         <v>REQ-012</v>
       </c>
       <c r="B13" t="str">
-        <v>Structuration données</v>
+        <v>IA &amp; Génération</v>
       </c>
       <c r="C13" t="str">
-        <v>Modèle Document</v>
+        <v>Prompt dynamique contextuel</v>
       </c>
       <c r="D13" t="str">
-        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
+        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
       </c>
       <c r="E13" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F13" t="str">
         <v>Complété</v>
       </c>
       <c r="G13" t="str">
-        <v>REQ-002</v>
+        <v>REQ-007</v>
       </c>
       <c r="H13" t="str">
-        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
+        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
       </c>
       <c r="I13" t="str">
-        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
+        <v>Zod validation sur count (1-10), language (fr/en)</v>
       </c>
     </row>
     <row r="14">
@@ -795,10 +795,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C14" t="str">
-        <v>Modèle Interviewé</v>
+        <v>Modèle Document</v>
       </c>
       <c r="D14" t="str">
-        <v>Nom complet, rôle, lié à campaign</v>
+        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
       </c>
       <c r="E14" t="str">
         <v>P0</v>
@@ -810,10 +810,10 @@
         <v>REQ-002</v>
       </c>
       <c r="H14" t="str">
-        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
+        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
       </c>
       <c r="I14" t="str">
-        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
+        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
       </c>
     </row>
     <row r="15">
@@ -824,10 +824,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C15" t="str">
-        <v>Modèle Note d'entretien</v>
+        <v>Modèle Interviewé</v>
       </c>
       <c r="D15" t="str">
-        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
+        <v>Nom complet, rôle, lié à campaign</v>
       </c>
       <c r="E15" t="str">
         <v>P0</v>
@@ -836,13 +836,13 @@
         <v>Complété</v>
       </c>
       <c r="G15" t="str">
-        <v>REQ-004, REQ-013</v>
+        <v>REQ-002</v>
       </c>
       <c r="H15" t="str">
-        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
+        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
       </c>
       <c r="I15" t="str">
-        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
+        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
       </c>
     </row>
     <row r="16">
@@ -853,25 +853,25 @@
         <v>Structuration données</v>
       </c>
       <c r="C16" t="str">
-        <v>Matrice de conformité</v>
+        <v>Modèle Note d'entretien</v>
       </c>
       <c r="D16" t="str">
-        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
+        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
       </c>
       <c r="E16" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F16" t="str">
         <v>Complété</v>
       </c>
       <c r="G16" t="str">
-        <v>REQ-014</v>
+        <v>REQ-005, REQ-014</v>
       </c>
       <c r="H16" t="str">
-        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
+        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
       </c>
       <c r="I16" t="str">
-        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
+        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
       </c>
     </row>
     <row r="17">
@@ -882,10 +882,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C17" t="str">
-        <v>Configuration Métriques</v>
+        <v>Matrice de conformité</v>
       </c>
       <c r="D17" t="str">
-        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
+        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
       </c>
       <c r="E17" t="str">
         <v>P1</v>
@@ -894,13 +894,13 @@
         <v>Complété</v>
       </c>
       <c r="G17" t="str">
-        <v>REQ-002</v>
+        <v>REQ-015</v>
       </c>
       <c r="H17" t="str">
-        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
+        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
       </c>
       <c r="I17" t="str">
-        <v>Format texte (ex: '1-5') pour flexibilité</v>
+        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
       </c>
     </row>
     <row r="18">
@@ -908,13 +908,13 @@
         <v>REQ-017</v>
       </c>
       <c r="B18" t="str">
-        <v>Audit &amp; Traçabilité</v>
+        <v>Structuration données</v>
       </c>
       <c r="C18" t="str">
-        <v>Audit Log complet</v>
+        <v>Configuration Métriques</v>
       </c>
       <c r="D18" t="str">
-        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
+        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
       </c>
       <c r="E18" t="str">
         <v>P1</v>
@@ -923,13 +923,13 @@
         <v>Complété</v>
       </c>
       <c r="G18" t="str">
-        <v>REQ-002, REQ-029</v>
+        <v>REQ-002</v>
       </c>
       <c r="H18" t="str">
-        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
+        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
       </c>
       <c r="I18" t="str">
-        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
+        <v>Format texte (ex: '1-5') pour flexibilité</v>
       </c>
     </row>
     <row r="19">
@@ -940,10 +940,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C19" t="str">
-        <v>Filtrage logs par période</v>
+        <v>Audit Log complet</v>
       </c>
       <c r="D19" t="str">
-        <v>Vue 7j, 30j, tout (by date range filter)</v>
+        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
       </c>
       <c r="E19" t="str">
         <v>P1</v>
@@ -952,13 +952,13 @@
         <v>Complété</v>
       </c>
       <c r="G19" t="str">
-        <v>REQ-017</v>
+        <v>REQ-002, REQ-030</v>
       </c>
       <c r="H19" t="str">
-        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
+        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
       </c>
       <c r="I19" t="str">
-        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
+        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
       </c>
     </row>
     <row r="20">
@@ -969,10 +969,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C20" t="str">
-        <v>Filtrage logs par action</v>
+        <v>Filtrage logs par période</v>
       </c>
       <c r="D20" t="str">
-        <v>Filter sur type d'action (campaign.created, etc.)</v>
+        <v>Vue 7j, 30j, tout (by date range filter)</v>
       </c>
       <c r="E20" t="str">
         <v>P1</v>
@@ -981,13 +981,13 @@
         <v>Complété</v>
       </c>
       <c r="G20" t="str">
-        <v>REQ-017</v>
+        <v>REQ-018</v>
       </c>
       <c r="H20" t="str">
-        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
+        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
       </c>
       <c r="I20" t="str">
-        <v>Enum actions découvertes dynamiquement from logs</v>
+        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
       </c>
     </row>
     <row r="21">
@@ -995,28 +995,28 @@
         <v>REQ-020</v>
       </c>
       <c r="B21" t="str">
-        <v>Rapports &amp; Exports</v>
+        <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C21" t="str">
-        <v>Export DOCX</v>
+        <v>Filtrage logs par action</v>
       </c>
       <c r="D21" t="str">
-        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
+        <v>Filter sur type d'action (campaign.created, etc.)</v>
       </c>
       <c r="E21" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F21" t="str">
         <v>Complété</v>
       </c>
       <c r="G21" t="str">
-        <v>REQ-005, REQ-015</v>
+        <v>REQ-018</v>
       </c>
       <c r="H21" t="str">
-        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
+        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
       </c>
       <c r="I21" t="str">
-        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
+        <v>Enum actions découvertes dynamiquement from logs</v>
       </c>
     </row>
     <row r="22">
@@ -1027,10 +1027,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C22" t="str">
-        <v>Export CSV</v>
+        <v>Export DOCX</v>
       </c>
       <c r="D22" t="str">
-        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
+        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
       </c>
       <c r="E22" t="str">
         <v>P2</v>
@@ -1039,13 +1039,13 @@
         <v>Complété</v>
       </c>
       <c r="G22" t="str">
-        <v>REQ-015, REQ-017</v>
+        <v>REQ-006, REQ-016</v>
       </c>
       <c r="H22" t="str">
-        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
+        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
       </c>
       <c r="I22" t="str">
-        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
+        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
       </c>
     </row>
     <row r="23">
@@ -1056,10 +1056,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C23" t="str">
-        <v>Gestion des rapports</v>
+        <v>Export CSV</v>
       </c>
       <c r="D23" t="str">
-        <v>Stocker rapports générés avec titre, date gen, version</v>
+        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
       </c>
       <c r="E23" t="str">
         <v>P2</v>
@@ -1068,13 +1068,13 @@
         <v>Complété</v>
       </c>
       <c r="G23" t="str">
-        <v>REQ-020, REQ-021</v>
+        <v>REQ-016, REQ-018</v>
       </c>
       <c r="H23" t="str">
-        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
+        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
       </c>
       <c r="I23" t="str">
-        <v>Récupérable dans UI, archivé pour traçabilité</v>
+        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
       </c>
     </row>
     <row r="24">
@@ -1082,28 +1082,28 @@
         <v>REQ-023</v>
       </c>
       <c r="B24" t="str">
-        <v>Dashboard &amp; Visualisation</v>
+        <v>Rapports &amp; Exports</v>
       </c>
       <c r="C24" t="str">
-        <v>KPIs essentiels</v>
+        <v>Gestion des rapports</v>
       </c>
       <c r="D24" t="str">
-        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
+        <v>Stocker rapports générés avec titre, date gen, version</v>
       </c>
       <c r="E24" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F24" t="str">
         <v>Complété</v>
       </c>
       <c r="G24" t="str">
-        <v>REQ-012, REQ-013, REQ-014</v>
+        <v>REQ-021, REQ-022</v>
       </c>
       <c r="H24" t="str">
-        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
+        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
       </c>
       <c r="I24" t="str">
-        <v>Affiché en gros chiffres zone haute dashboard</v>
+        <v>Récupérable dans UI, archivé pour traçabilité</v>
       </c>
     </row>
     <row r="25">
@@ -1114,25 +1114,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C25" t="str">
-        <v>Matrice de conformité interactive</v>
+        <v>KPIs essentiels</v>
       </c>
       <c r="D25" t="str">
-        <v>Tableau avec % conformité par criterion, tri/filtre</v>
+        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
       </c>
       <c r="E25" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F25" t="str">
         <v>Complété</v>
       </c>
       <c r="G25" t="str">
-        <v>REQ-015</v>
+        <v>REQ-013, REQ-014, REQ-015</v>
       </c>
       <c r="H25" t="str">
-        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
+        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
       </c>
       <c r="I25" t="str">
-        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
+        <v>Affiché en gros chiffres zone haute dashboard</v>
       </c>
     </row>
     <row r="26">
@@ -1143,25 +1143,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C26" t="str">
-        <v>Graphiques optionnels (futur)</v>
+        <v>Matrice de conformité interactive</v>
       </c>
       <c r="D26" t="str">
-        <v>Tendances audit timeline, pie charts conformity domains</v>
+        <v>Tableau avec % conformité par criterion, tri/filtre</v>
       </c>
       <c r="E26" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="F26" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G26" t="str">
-        <v>REQ-023</v>
+        <v>REQ-016</v>
       </c>
       <c r="H26" t="str">
-        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
+        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
       </c>
       <c r="I26" t="str">
-        <v>MVP n'a pas graphiques, architecture prête pour.</v>
+        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
       </c>
     </row>
     <row r="27">
@@ -1169,28 +1169,28 @@
         <v>REQ-026</v>
       </c>
       <c r="B27" t="str">
-        <v>Configuration &amp; Flexibilité</v>
+        <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C27" t="str">
-        <v>Support multilingue</v>
+        <v>Graphiques optionnels (futur)</v>
       </c>
       <c r="D27" t="str">
-        <v>FR et EN, sélection par campaign</v>
+        <v>Tendances audit timeline, pie charts conformity domains</v>
       </c>
       <c r="E27" t="str">
-        <v>P1</v>
+        <v>P3</v>
       </c>
       <c r="F27" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G27" t="str">
-        <v>REQ-029</v>
+        <v>REQ-024</v>
       </c>
       <c r="H27" t="str">
-        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
+        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
       </c>
       <c r="I27" t="str">
-        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
+        <v>MVP n'a pas graphiques, architecture prête pour.</v>
       </c>
     </row>
     <row r="28">
@@ -1201,10 +1201,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C28" t="str">
-        <v>Modèle Ollama configurable</v>
+        <v>Support multilingue</v>
       </c>
       <c r="D28" t="str">
-        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
+        <v>FR et EN, sélection par campaign</v>
       </c>
       <c r="E28" t="str">
         <v>P1</v>
@@ -1213,13 +1213,13 @@
         <v>Complété</v>
       </c>
       <c r="G28" t="str">
-        <v>REQ-008</v>
+        <v>REQ-030</v>
       </c>
       <c r="H28" t="str">
-        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
+        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
       </c>
       <c r="I28" t="str">
-        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
+        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
       </c>
     </row>
     <row r="29">
@@ -1230,10 +1230,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C29" t="str">
-        <v>OpenAI optionnel</v>
+        <v>Modèle Ollama configurable</v>
       </c>
       <c r="D29" t="str">
-        <v>API key via .env, fallback auto Ollama si absent</v>
+        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
       </c>
       <c r="E29" t="str">
         <v>P1</v>
@@ -1242,13 +1242,13 @@
         <v>Complété</v>
       </c>
       <c r="G29" t="str">
-        <v>REQ-029</v>
+        <v>REQ-009</v>
       </c>
       <c r="H29" t="str">
-        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
+        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
       </c>
       <c r="I29" t="str">
-        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
+        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
       </c>
     </row>
     <row r="30">
@@ -1259,25 +1259,25 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C30" t="str">
-        <v>Thèmes personnalisés</v>
+        <v>OpenAI optionnel</v>
       </c>
       <c r="D30" t="str">
-        <v>Texte libre pour documents et questions</v>
+        <v>API key via .env, fallback auto Ollama si absent</v>
       </c>
       <c r="E30" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F30" t="str">
         <v>Complété</v>
       </c>
       <c r="G30" t="str">
-        <v>-</v>
+        <v>REQ-030</v>
       </c>
       <c r="H30" t="str">
-        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
+        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
       </c>
       <c r="I30" t="str">
-        <v>Permet flexibilité sur domaines audit custom</v>
+        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
       </c>
     </row>
     <row r="31">
@@ -1285,16 +1285,16 @@
         <v>REQ-030</v>
       </c>
       <c r="B31" t="str">
-        <v>Infrastructure &amp; Déploiement</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C31" t="str">
-        <v>Offline-first capability</v>
+        <v>Thèmes personnalisés</v>
       </c>
       <c r="D31" t="str">
-        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
+        <v>Texte libre pour documents et questions</v>
       </c>
       <c r="E31" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F31" t="str">
         <v>Complété</v>
@@ -1303,10 +1303,10 @@
         <v>-</v>
       </c>
       <c r="H31" t="str">
-        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
+        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
       </c>
       <c r="I31" t="str">
-        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
+        <v>Permet flexibilité sur domaines audit custom</v>
       </c>
     </row>
     <row r="32">
@@ -1317,25 +1317,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C32" t="str">
-        <v>Automation PowerShell</v>
+        <v>Offline-first capability</v>
       </c>
       <c r="D32" t="str">
-        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
+        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
       </c>
       <c r="E32" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F32" t="str">
         <v>Complété</v>
       </c>
       <c r="G32" t="str">
-        <v>REQ-027, REQ-030</v>
+        <v>-</v>
       </c>
       <c r="H32" t="str">
-        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
+        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
       </c>
       <c r="I32" t="str">
-        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
+        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
       </c>
     </row>
     <row r="33">
@@ -1346,25 +1346,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C33" t="str">
-        <v>Versionning Git &amp; GitHub</v>
+        <v>Automation PowerShell</v>
       </c>
       <c r="D33" t="str">
-        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
+        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
       </c>
       <c r="E33" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F33" t="str">
         <v>Complété</v>
       </c>
       <c r="G33" t="str">
-        <v>REQ-006, REQ-030</v>
+        <v>REQ-028, REQ-031</v>
       </c>
       <c r="H33" t="str">
-        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
+        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
       </c>
       <c r="I33" t="str">
-        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
+        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
       </c>
     </row>
     <row r="34">
@@ -1375,25 +1375,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C34" t="str">
-        <v>API REST Fastify</v>
+        <v>Versionning Git &amp; GitHub</v>
       </c>
       <c r="D34" t="str">
-        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
+        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
       </c>
       <c r="E34" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F34" t="str">
         <v>Complété</v>
       </c>
       <c r="G34" t="str">
-        <v>REQ-012, REQ-030</v>
+        <v>REQ-007, REQ-031</v>
       </c>
       <c r="H34" t="str">
-        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
+        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
       </c>
       <c r="I34" t="str">
-        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
+        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
       </c>
     </row>
     <row r="35">
@@ -1401,28 +1401,28 @@
         <v>REQ-034</v>
       </c>
       <c r="B35" t="str">
-        <v>UI/UX</v>
+        <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C35" t="str">
-        <v>UI React + TypeScript + Vite</v>
+        <v>API REST Fastify</v>
       </c>
       <c r="D35" t="str">
-        <v>Bundling optimisé, HMR dev mode</v>
+        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
       </c>
       <c r="E35" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F35" t="str">
         <v>Complété</v>
       </c>
       <c r="G35" t="str">
-        <v>REQ-016, REQ-030</v>
+        <v>REQ-013, REQ-031</v>
       </c>
       <c r="H35" t="str">
-        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
+        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
       </c>
       <c r="I35" t="str">
-        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
+        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
       </c>
     </row>
     <row r="36">
@@ -1433,10 +1433,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C36" t="str">
-        <v>Configuration IA section</v>
+        <v>UI React + TypeScript + Vite</v>
       </c>
       <c r="D36" t="str">
-        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
+        <v>Bundling optimisé, HMR dev mode</v>
       </c>
       <c r="E36" t="str">
         <v>P1</v>
@@ -1445,13 +1445,13 @@
         <v>Complété</v>
       </c>
       <c r="G36" t="str">
-        <v>REQ-023, REQ-030</v>
+        <v>REQ-017, REQ-031</v>
       </c>
       <c r="H36" t="str">
-        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
+        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
       </c>
       <c r="I36" t="str">
-        <v>UX: clair et accessible, pas scroll nécessaire</v>
+        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
       </c>
     </row>
     <row r="37">
@@ -1462,10 +1462,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C37" t="str">
-        <v>Génération questions section</v>
+        <v>Configuration IA section</v>
       </c>
       <c r="D37" t="str">
-        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
+        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
       </c>
       <c r="E37" t="str">
         <v>P1</v>
@@ -1474,13 +1474,13 @@
         <v>Complété</v>
       </c>
       <c r="G37" t="str">
-        <v>REQ-013, REQ-014, REQ-030</v>
+        <v>REQ-024, REQ-031</v>
       </c>
       <c r="H37" t="str">
-        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
+        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
       </c>
       <c r="I37" t="str">
-        <v>État uploadingReferential: loading indicator, disabled submit</v>
+        <v>UX: clair et accessible, pas scroll nécessaire</v>
       </c>
     </row>
     <row r="38">
@@ -1491,10 +1491,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C38" t="str">
-        <v>Référentiel documentaire section</v>
+        <v>Génération questions section</v>
       </c>
       <c r="D38" t="str">
-        <v>Ajouter document avec métas, liste affichée</v>
+        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
       </c>
       <c r="E38" t="str">
         <v>P1</v>
@@ -1503,13 +1503,13 @@
         <v>Complété</v>
       </c>
       <c r="G38" t="str">
-        <v>REQ-018, REQ-019, REQ-030</v>
+        <v>REQ-014, REQ-015, REQ-031</v>
       </c>
       <c r="H38" t="str">
-        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
+        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
       </c>
       <c r="I38" t="str">
-        <v>Erreurs affichées, success feedback, état documentS refresh</v>
+        <v>État uploadingReferential: loading indicator, disabled submit</v>
       </c>
     </row>
     <row r="39">
@@ -1520,10 +1520,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C39" t="str">
-        <v>Échelles métriques config</v>
+        <v>Référentiel documentaire section</v>
       </c>
       <c r="D39" t="str">
-        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
+        <v>Ajouter document avec métas, liste affichée</v>
       </c>
       <c r="E39" t="str">
         <v>P1</v>
@@ -1532,13 +1532,13 @@
         <v>Complété</v>
       </c>
       <c r="G39" t="str">
-        <v>REQ-020, REQ-021, REQ-030</v>
+        <v>REQ-019, REQ-020, REQ-031</v>
       </c>
       <c r="H39" t="str">
-        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
+        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
       </c>
       <c r="I39" t="str">
-        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
+        <v>Erreurs affichées, success feedback, état documentS refresh</v>
       </c>
     </row>
     <row r="40">
@@ -1549,10 +1549,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C40" t="str">
-        <v>Dashboard avec KPIs</v>
+        <v>Échelles métriques config</v>
       </c>
       <c r="D40" t="str">
-        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
+        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
       </c>
       <c r="E40" t="str">
         <v>P1</v>
@@ -1561,13 +1561,13 @@
         <v>Complété</v>
       </c>
       <c r="G40" t="str">
-        <v>-</v>
+        <v>REQ-021, REQ-022, REQ-031</v>
       </c>
       <c r="H40" t="str">
-        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
+        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
       </c>
       <c r="I40" t="str">
-        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
+        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
       </c>
     </row>
     <row r="41">
@@ -1578,10 +1578,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C41" t="str">
-        <v>Gestion entretiens</v>
+        <v>Dashboard avec KPIs</v>
       </c>
       <c r="D41" t="str">
-        <v>Interviewés, notes questions, scoring intégré</v>
+        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
       </c>
       <c r="E41" t="str">
         <v>P1</v>
@@ -1593,10 +1593,10 @@
         <v>-</v>
       </c>
       <c r="H41" t="str">
-        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
+        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
       </c>
       <c r="I41" t="str">
-        <v>Chaque note liée criterion + interviewee + score optionnel</v>
+        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
       </c>
     </row>
     <row r="42">
@@ -1607,10 +1607,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C42" t="str">
-        <v>Audit log viewer</v>
+        <v>Gestion entretiens</v>
       </c>
       <c r="D42" t="str">
-        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
+        <v>Interviewés, notes questions, scoring intégré</v>
       </c>
       <c r="E42" t="str">
         <v>P1</v>
@@ -1619,13 +1619,13 @@
         <v>Complété</v>
       </c>
       <c r="G42" t="str">
-        <v>REQ-040</v>
+        <v>-</v>
       </c>
       <c r="H42" t="str">
-        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
+        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
       </c>
       <c r="I42" t="str">
-        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
+        <v>Chaque note liée criterion + interviewee + score optionnel</v>
       </c>
     </row>
     <row r="43">
@@ -1636,25 +1636,25 @@
         <v>UI/UX</v>
       </c>
       <c r="C43" t="str">
-        <v>Export buttons</v>
+        <v>Audit log viewer</v>
       </c>
       <c r="D43" t="str">
-        <v>Boutons DOCX et CSV téléchargement</v>
+        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
       </c>
       <c r="E43" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F43" t="str">
         <v>Complété</v>
       </c>
       <c r="G43" t="str">
-        <v>-</v>
+        <v>REQ-041</v>
       </c>
       <c r="H43" t="str">
-        <v>POST /export-report et /export-csv. browser Blob download.</v>
+        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
       </c>
       <c r="I43" t="str">
-        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
       </c>
     </row>
     <row r="44">
@@ -1662,13 +1662,13 @@
         <v>REQ-043</v>
       </c>
       <c r="B44" t="str">
-        <v>Persévérance &amp; Facilité</v>
+        <v>UI/UX</v>
       </c>
       <c r="C44" t="str">
-        <v>Documentation complète</v>
+        <v>Export buttons</v>
       </c>
       <c r="D44" t="str">
-        <v>Setup guides, quickstart, git manual, examples références</v>
+        <v>Boutons DOCX et CSV téléchargement</v>
       </c>
       <c r="E44" t="str">
         <v>P2</v>
@@ -1680,13 +1680,13 @@
         <v>-</v>
       </c>
       <c r="H44" t="str">
-        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
+        <v>POST /export-report et /export-csv. browser Blob download.</v>
       </c>
       <c r="I44" t="str">
-        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
+        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+      </c>
+    </row>
+    <row r="45">
       <c r="A45" t="str">
         <v>REQ-044</v>
       </c>
@@ -1694,10 +1694,10 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C45" t="str">
-        <v>One-command installation</v>
+        <v>Documentation complète</v>
       </c>
       <c r="D45" t="str">
-        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+        <v>Setup guides, quickstart, git manual, examples références</v>
       </c>
       <c r="E45" t="str">
         <v>P2</v>
@@ -1708,12 +1708,11 @@
       <c r="G45" t="str">
         <v>-</v>
       </c>
-      <c r="H45" t="str" xml:space="preserve">
-        <v xml:space="preserve">.
- install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      <c r="H45" t="str">
+        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
       </c>
       <c r="I45" t="str">
-        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -1724,41 +1723,42 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C46" t="str">
+        <v>One-command installation</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+      </c>
+      <c r="E46" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G46" t="str">
+        <v>-</v>
+      </c>
+      <c r="H46" t="str" xml:space="preserve">
+        <v xml:space="preserve">.
+ install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      </c>
+      <c r="I46" t="str">
+        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
+        <v>REQ-046</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C47" t="str">
         <v>One-command launch</v>
       </c>
-      <c r="D46" t="str" xml:space="preserve">
+      <c r="D47" t="str" xml:space="preserve">
         <v xml:space="preserve">npm run dev ou .
 start-rubis.ps1 pour lancer tout</v>
       </c>
-      <c r="E46" t="str">
-        <v>P2</v>
-      </c>
-      <c r="F46" t="str">
-        <v>Complété</v>
-      </c>
-      <c r="G46" t="str">
-        <v>-</v>
-      </c>
-      <c r="H46" t="str">
-        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
-      </c>
-      <c r="I46" t="str">
-        <v>Détection auto erreurs, log output lisible</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>REQ-046</v>
-      </c>
-      <c r="B47" t="str">
-        <v>Persévérance &amp; Facilité</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Clear error messages</v>
-      </c>
-      <c r="D47" t="str">
-        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
-      </c>
       <c r="E47" t="str">
         <v>P2</v>
       </c>
@@ -1769,10 +1769,10 @@
         <v>-</v>
       </c>
       <c r="H47" t="str">
-        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
       </c>
       <c r="I47" t="str">
-        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+        <v>Détection auto erreurs, log output lisible</v>
       </c>
     </row>
     <row r="48">
@@ -1783,30 +1783,59 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C48" t="str">
-        <v>Roadmap versioning</v>
+        <v>Clear error messages</v>
       </c>
       <c r="D48" t="str">
-        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
       </c>
       <c r="E48" t="str">
         <v>P2</v>
       </c>
       <c r="F48" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G48" t="str">
         <v>-</v>
       </c>
       <c r="H48" t="str">
+        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>REQ-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Roadmap versioning</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+      </c>
+      <c r="E49" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Planifié</v>
+      </c>
+      <c r="G49" t="str">
+        <v>-</v>
+      </c>
+      <c r="H49" t="str">
         <v>Créer ROADMAP.xlsx avec specs, priorités, statuts, directives implémentation.</v>
       </c>
-      <c r="I48" t="str">
+      <c r="I49" t="str">
         <v>À committé dans git, mis à jour post-MVP pour v2 features</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I48"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I49"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Add automatic criteria extraction from referential to roadmap (REQ-006)
- New specification: Extraction automatique des critères depuis référentiel
- Domain: IA & Génération
- Priority: P1
- Status: Planifié
- Features: IA parse document référentiel (ISO27001, PASSI, etc.)
- Extracts: code, titre, thème, description for all requirements/controls
- Example: ISO27001 → auto-extract A.5.1 to A.18.2 (93 controls)
- UI: upload doc + preview + validate before import
- Dependencies: REQ-005 (Critères), REQ-003 (Référentiels), REQ-031 (API)
- Total: 49 specifications (was 48)
- Massive time savings vs manual entry
</commit_message>
<xml_diff>
--- a/ROADMAP.xlsx
+++ b/ROADMAP.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I50"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -546,7 +546,7 @@
         <v>Planifié</v>
       </c>
       <c r="G5" t="str">
-        <v>REQ-003, REQ-030</v>
+        <v>REQ-003, REQ-031</v>
       </c>
       <c r="H5" t="str">
         <v>Section admin protégée. CRUD référentiels: POST/PUT/DELETE /admin/referentials. Stockage db.data.referentials avec {id, name, category, description, isActive}. UI table éditable avec formulaire modal.</v>
@@ -589,28 +589,28 @@
         <v>REQ-006</v>
       </c>
       <c r="B7" t="str">
-        <v>Cœur métier</v>
+        <v>IA &amp; Génération</v>
       </c>
       <c r="C7" t="str">
-        <v>Génération de questions</v>
+        <v>Extraction automatique des critères depuis référentiel</v>
       </c>
       <c r="D7" t="str">
-        <v>Questions avec text, guidance, theme générées dynamiquement</v>
+        <v>IA parse le document référentiel fourni (PDF/Excel) et extrait automatiquement tous les critères/exigences avec code, titre, description</v>
       </c>
       <c r="E7" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F7" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G7" t="str">
-        <v>REQ-005</v>
+        <v>REQ-005, REQ-003, REQ-031</v>
       </c>
       <c r="H7" t="str">
-        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
+        <v>POST /extract-criteria-from-referential. Multipart upload. Parser identifie structure (ex: ISO27001 A.5.1, A.5.2...). LLM extrait: {code, title, theme, description}. Batch insert criteria. UI: upload doc + bouton 'Extraire critères', preview avant validation.</v>
       </c>
       <c r="I7" t="str">
-        <v>Peut être depuis template ou IA (voir section IA)</v>
+        <v>Exemple: ISO27001 → extraire A.5.1 à A.18.2 (93 contrôles). PASSI → extraire exigences numérotées. Gain temps énorme vs saisie manuelle. Validation humaine optionnelle avant import.</v>
       </c>
     </row>
     <row r="8">
@@ -618,16 +618,16 @@
         <v>REQ-007</v>
       </c>
       <c r="B8" t="str">
-        <v>IA &amp; Génération</v>
+        <v>Cœur métier</v>
       </c>
       <c r="C8" t="str">
-        <v>Génération depuis référentiel</v>
+        <v>Génération de questions</v>
       </c>
       <c r="D8" t="str">
-        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
+        <v>Questions avec text, guidance, theme générées dynamiquement</v>
       </c>
       <c r="E8" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F8" t="str">
         <v>Complété</v>
@@ -636,10 +636,10 @@
         <v>REQ-005</v>
       </c>
       <c r="H8" t="str">
-        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
+        <v>POST /question, GET /questions. Schéma Zod pour validation stricte.</v>
       </c>
       <c r="I8" t="str">
-        <v>Limite 50KB texte extrait pour perf API</v>
+        <v>Peut être depuis template ou IA (voir section IA)</v>
       </c>
     </row>
     <row r="9">
@@ -650,10 +650,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C9" t="str">
-        <v>Dual AI strategy - OpenAI</v>
+        <v>Génération depuis référentiel</v>
       </c>
       <c r="D9" t="str">
-        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
+        <v>Parser PDF ou Excel, extraire texte, passer à IA pour générer questions</v>
       </c>
       <c r="E9" t="str">
         <v>P1</v>
@@ -662,13 +662,13 @@
         <v>Complété</v>
       </c>
       <c r="G9" t="str">
-        <v>REQ-030</v>
+        <v>REQ-006</v>
       </c>
       <c r="H9" t="str">
-        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
+        <v>POST /generate-questions-from-referential. Multipart form. parseReferentialFile() en services/referentialParser.ts</v>
       </c>
       <c r="I9" t="str">
-        <v>Fallback si OPENAI_API_KEY absent</v>
+        <v>Limite 50KB texte extrait pour perf API</v>
       </c>
     </row>
     <row r="10">
@@ -679,10 +679,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C10" t="str">
-        <v>Dual AI strategy - Ollama local</v>
+        <v>Dual AI strategy - OpenAI</v>
       </c>
       <c r="D10" t="str">
-        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
+        <v>Intégration GPT-4o pour génération rapide et haute qualité</v>
       </c>
       <c r="E10" t="str">
         <v>P1</v>
@@ -691,13 +691,13 @@
         <v>Complété</v>
       </c>
       <c r="G10" t="str">
-        <v>REQ-030</v>
+        <v>REQ-031</v>
       </c>
       <c r="H10" t="str">
-        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
+        <v>generateQuestionsFromOpenAI() dans openai.ts. OpenAI client avec apiKey depuis .env</v>
       </c>
       <c r="I10" t="str">
-        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
+        <v>Fallback si OPENAI_API_KEY absent</v>
       </c>
     </row>
     <row r="11">
@@ -708,10 +708,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C11" t="str">
-        <v>Model switching UI</v>
+        <v>Dual AI strategy - Ollama local</v>
       </c>
       <c r="D11" t="str">
-        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
+        <v>Ollama + Mistral/Gemma3 pour mode offline-first sur éliteBook</v>
       </c>
       <c r="E11" t="str">
         <v>P1</v>
@@ -720,13 +720,13 @@
         <v>Complété</v>
       </c>
       <c r="G11" t="str">
-        <v>REQ-008, REQ-009</v>
+        <v>REQ-031</v>
       </c>
       <c r="H11" t="str">
-        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
+        <v>generateQuestionsFromOllama() fetch to localhost:11434/api/generate. checkOllamaAvailable() avec timeout 2s</v>
       </c>
       <c r="I11" t="str">
-        <v>Changement runtime, pas besoin restart API</v>
+        <v>Auto-détection Ollama, fallback depuis OpenAI si non dispo</v>
       </c>
     </row>
     <row r="12">
@@ -737,10 +737,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C12" t="str">
-        <v>Parsing référentiel multi-format</v>
+        <v>Model switching UI</v>
       </c>
       <c r="D12" t="str">
-        <v>Support PDF et Excel avec extraction de texte</v>
+        <v>Permuter entre mistral et gemma3:4b directement dans l'appli</v>
       </c>
       <c r="E12" t="str">
         <v>P1</v>
@@ -749,13 +749,13 @@
         <v>Complété</v>
       </c>
       <c r="G12" t="str">
-        <v>REQ-007</v>
+        <v>REQ-009, REQ-010</v>
       </c>
       <c r="H12" t="str">
-        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
+        <v>GET/POST /config endpoints. État currentOllamaModel dans server.ts. Boutons UI dans App.tsx 'Configuration IA'</v>
       </c>
       <c r="I12" t="str">
-        <v>Gère encodages UTF-8, caractères spéciaux</v>
+        <v>Changement runtime, pas besoin restart API</v>
       </c>
     </row>
     <row r="13">
@@ -766,10 +766,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C13" t="str">
-        <v>Prompt dynamique contextuel</v>
+        <v>Parsing référentiel multi-format</v>
       </c>
       <c r="D13" t="str">
-        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
+        <v>Support PDF et Excel avec extraction de texte</v>
       </c>
       <c r="E13" t="str">
         <v>P1</v>
@@ -778,13 +778,13 @@
         <v>Complété</v>
       </c>
       <c r="G13" t="str">
-        <v>REQ-007</v>
+        <v>REQ-008</v>
       </c>
       <c r="H13" t="str">
-        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
+        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
       </c>
       <c r="I13" t="str">
-        <v>Zod validation sur count (1-10), language (fr/en)</v>
+        <v>Gère encodages UTF-8, caractères spéciaux</v>
       </c>
     </row>
     <row r="14">
@@ -792,28 +792,28 @@
         <v>REQ-013</v>
       </c>
       <c r="B14" t="str">
-        <v>Structuration données</v>
+        <v>IA &amp; Génération</v>
       </c>
       <c r="C14" t="str">
-        <v>Modèle Document</v>
+        <v>Prompt dynamique contextuel</v>
       </c>
       <c r="D14" t="str">
-        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
+        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
       </c>
       <c r="E14" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F14" t="str">
         <v>Complété</v>
       </c>
       <c r="G14" t="str">
-        <v>REQ-002</v>
+        <v>REQ-008</v>
       </c>
       <c r="H14" t="str">
-        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
+        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
       </c>
       <c r="I14" t="str">
-        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
+        <v>Zod validation sur count (1-10), language (fr/en)</v>
       </c>
     </row>
     <row r="15">
@@ -824,10 +824,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C15" t="str">
-        <v>Modèle Interviewé</v>
+        <v>Modèle Document</v>
       </c>
       <c r="D15" t="str">
-        <v>Nom complet, rôle, lié à campaign</v>
+        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
       </c>
       <c r="E15" t="str">
         <v>P0</v>
@@ -839,10 +839,10 @@
         <v>REQ-002</v>
       </c>
       <c r="H15" t="str">
-        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
+        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
       </c>
       <c r="I15" t="str">
-        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
+        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
       </c>
     </row>
     <row r="16">
@@ -853,10 +853,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C16" t="str">
-        <v>Modèle Note d'entretien</v>
+        <v>Modèle Interviewé</v>
       </c>
       <c r="D16" t="str">
-        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
+        <v>Nom complet, rôle, lié à campaign</v>
       </c>
       <c r="E16" t="str">
         <v>P0</v>
@@ -865,13 +865,13 @@
         <v>Complété</v>
       </c>
       <c r="G16" t="str">
-        <v>REQ-005, REQ-014</v>
+        <v>REQ-002</v>
       </c>
       <c r="H16" t="str">
-        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
+        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
       </c>
       <c r="I16" t="str">
-        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
+        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
       </c>
     </row>
     <row r="17">
@@ -882,25 +882,25 @@
         <v>Structuration données</v>
       </c>
       <c r="C17" t="str">
-        <v>Matrice de conformité</v>
+        <v>Modèle Note d'entretien</v>
       </c>
       <c r="D17" t="str">
-        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
+        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
       </c>
       <c r="E17" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F17" t="str">
         <v>Complété</v>
       </c>
       <c r="G17" t="str">
-        <v>REQ-015</v>
+        <v>REQ-005, REQ-015</v>
       </c>
       <c r="H17" t="str">
-        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
+        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
       </c>
       <c r="I17" t="str">
-        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
+        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
       </c>
     </row>
     <row r="18">
@@ -911,10 +911,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C18" t="str">
-        <v>Configuration Métriques</v>
+        <v>Matrice de conformité</v>
       </c>
       <c r="D18" t="str">
-        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
+        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
       </c>
       <c r="E18" t="str">
         <v>P1</v>
@@ -923,13 +923,13 @@
         <v>Complété</v>
       </c>
       <c r="G18" t="str">
-        <v>REQ-002</v>
+        <v>REQ-016</v>
       </c>
       <c r="H18" t="str">
-        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
+        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
       </c>
       <c r="I18" t="str">
-        <v>Format texte (ex: '1-5') pour flexibilité</v>
+        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
       </c>
     </row>
     <row r="19">
@@ -937,13 +937,13 @@
         <v>REQ-018</v>
       </c>
       <c r="B19" t="str">
-        <v>Audit &amp; Traçabilité</v>
+        <v>Structuration données</v>
       </c>
       <c r="C19" t="str">
-        <v>Audit Log complet</v>
+        <v>Configuration Métriques</v>
       </c>
       <c r="D19" t="str">
-        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
+        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
       </c>
       <c r="E19" t="str">
         <v>P1</v>
@@ -952,13 +952,13 @@
         <v>Complété</v>
       </c>
       <c r="G19" t="str">
-        <v>REQ-002, REQ-030</v>
+        <v>REQ-002</v>
       </c>
       <c r="H19" t="str">
-        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
+        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
       </c>
       <c r="I19" t="str">
-        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
+        <v>Format texte (ex: '1-5') pour flexibilité</v>
       </c>
     </row>
     <row r="20">
@@ -969,10 +969,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C20" t="str">
-        <v>Filtrage logs par période</v>
+        <v>Audit Log complet</v>
       </c>
       <c r="D20" t="str">
-        <v>Vue 7j, 30j, tout (by date range filter)</v>
+        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
       </c>
       <c r="E20" t="str">
         <v>P1</v>
@@ -981,13 +981,13 @@
         <v>Complété</v>
       </c>
       <c r="G20" t="str">
-        <v>REQ-018</v>
+        <v>REQ-002, REQ-031</v>
       </c>
       <c r="H20" t="str">
-        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
+        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
       </c>
       <c r="I20" t="str">
-        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
+        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
       </c>
     </row>
     <row r="21">
@@ -998,10 +998,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C21" t="str">
-        <v>Filtrage logs par action</v>
+        <v>Filtrage logs par période</v>
       </c>
       <c r="D21" t="str">
-        <v>Filter sur type d'action (campaign.created, etc.)</v>
+        <v>Vue 7j, 30j, tout (by date range filter)</v>
       </c>
       <c r="E21" t="str">
         <v>P1</v>
@@ -1010,13 +1010,13 @@
         <v>Complété</v>
       </c>
       <c r="G21" t="str">
-        <v>REQ-018</v>
+        <v>REQ-019</v>
       </c>
       <c r="H21" t="str">
-        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
+        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
       </c>
       <c r="I21" t="str">
-        <v>Enum actions découvertes dynamiquement from logs</v>
+        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
       </c>
     </row>
     <row r="22">
@@ -1024,28 +1024,28 @@
         <v>REQ-021</v>
       </c>
       <c r="B22" t="str">
-        <v>Rapports &amp; Exports</v>
+        <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C22" t="str">
-        <v>Export DOCX</v>
+        <v>Filtrage logs par action</v>
       </c>
       <c r="D22" t="str">
-        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
+        <v>Filter sur type d'action (campaign.created, etc.)</v>
       </c>
       <c r="E22" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F22" t="str">
         <v>Complété</v>
       </c>
       <c r="G22" t="str">
-        <v>REQ-006, REQ-016</v>
+        <v>REQ-019</v>
       </c>
       <c r="H22" t="str">
-        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
+        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
       </c>
       <c r="I22" t="str">
-        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
+        <v>Enum actions découvertes dynamiquement from logs</v>
       </c>
     </row>
     <row r="23">
@@ -1056,10 +1056,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C23" t="str">
-        <v>Export CSV</v>
+        <v>Export DOCX</v>
       </c>
       <c r="D23" t="str">
-        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
+        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
       </c>
       <c r="E23" t="str">
         <v>P2</v>
@@ -1068,13 +1068,13 @@
         <v>Complété</v>
       </c>
       <c r="G23" t="str">
-        <v>REQ-016, REQ-018</v>
+        <v>REQ-007, REQ-017</v>
       </c>
       <c r="H23" t="str">
-        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
+        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
       </c>
       <c r="I23" t="str">
-        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
+        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
       </c>
     </row>
     <row r="24">
@@ -1085,10 +1085,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C24" t="str">
-        <v>Gestion des rapports</v>
+        <v>Export CSV</v>
       </c>
       <c r="D24" t="str">
-        <v>Stocker rapports générés avec titre, date gen, version</v>
+        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
       </c>
       <c r="E24" t="str">
         <v>P2</v>
@@ -1097,13 +1097,13 @@
         <v>Complété</v>
       </c>
       <c r="G24" t="str">
-        <v>REQ-021, REQ-022</v>
+        <v>REQ-017, REQ-019</v>
       </c>
       <c r="H24" t="str">
-        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
+        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
       </c>
       <c r="I24" t="str">
-        <v>Récupérable dans UI, archivé pour traçabilité</v>
+        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
       </c>
     </row>
     <row r="25">
@@ -1111,28 +1111,28 @@
         <v>REQ-024</v>
       </c>
       <c r="B25" t="str">
-        <v>Dashboard &amp; Visualisation</v>
+        <v>Rapports &amp; Exports</v>
       </c>
       <c r="C25" t="str">
-        <v>KPIs essentiels</v>
+        <v>Gestion des rapports</v>
       </c>
       <c r="D25" t="str">
-        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
+        <v>Stocker rapports générés avec titre, date gen, version</v>
       </c>
       <c r="E25" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F25" t="str">
         <v>Complété</v>
       </c>
       <c r="G25" t="str">
-        <v>REQ-013, REQ-014, REQ-015</v>
+        <v>REQ-022, REQ-023</v>
       </c>
       <c r="H25" t="str">
-        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
+        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
       </c>
       <c r="I25" t="str">
-        <v>Affiché en gros chiffres zone haute dashboard</v>
+        <v>Récupérable dans UI, archivé pour traçabilité</v>
       </c>
     </row>
     <row r="26">
@@ -1143,25 +1143,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C26" t="str">
-        <v>Matrice de conformité interactive</v>
+        <v>KPIs essentiels</v>
       </c>
       <c r="D26" t="str">
-        <v>Tableau avec % conformité par criterion, tri/filtre</v>
+        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
       </c>
       <c r="E26" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F26" t="str">
         <v>Complété</v>
       </c>
       <c r="G26" t="str">
-        <v>REQ-016</v>
+        <v>REQ-014, REQ-015, REQ-016</v>
       </c>
       <c r="H26" t="str">
-        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
+        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
       </c>
       <c r="I26" t="str">
-        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
+        <v>Affiché en gros chiffres zone haute dashboard</v>
       </c>
     </row>
     <row r="27">
@@ -1172,25 +1172,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C27" t="str">
-        <v>Graphiques optionnels (futur)</v>
+        <v>Matrice de conformité interactive</v>
       </c>
       <c r="D27" t="str">
-        <v>Tendances audit timeline, pie charts conformity domains</v>
+        <v>Tableau avec % conformité par criterion, tri/filtre</v>
       </c>
       <c r="E27" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="F27" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G27" t="str">
-        <v>REQ-024</v>
+        <v>REQ-017</v>
       </c>
       <c r="H27" t="str">
-        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
+        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
       </c>
       <c r="I27" t="str">
-        <v>MVP n'a pas graphiques, architecture prête pour.</v>
+        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
       </c>
     </row>
     <row r="28">
@@ -1198,28 +1198,28 @@
         <v>REQ-027</v>
       </c>
       <c r="B28" t="str">
-        <v>Configuration &amp; Flexibilité</v>
+        <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C28" t="str">
-        <v>Support multilingue</v>
+        <v>Graphiques optionnels (futur)</v>
       </c>
       <c r="D28" t="str">
-        <v>FR et EN, sélection par campaign</v>
+        <v>Tendances audit timeline, pie charts conformity domains</v>
       </c>
       <c r="E28" t="str">
-        <v>P1</v>
+        <v>P3</v>
       </c>
       <c r="F28" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G28" t="str">
-        <v>REQ-030</v>
+        <v>REQ-025</v>
       </c>
       <c r="H28" t="str">
-        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
+        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
       </c>
       <c r="I28" t="str">
-        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
+        <v>MVP n'a pas graphiques, architecture prête pour.</v>
       </c>
     </row>
     <row r="29">
@@ -1230,10 +1230,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C29" t="str">
-        <v>Modèle Ollama configurable</v>
+        <v>Support multilingue</v>
       </c>
       <c r="D29" t="str">
-        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
+        <v>FR et EN, sélection par campaign</v>
       </c>
       <c r="E29" t="str">
         <v>P1</v>
@@ -1242,13 +1242,13 @@
         <v>Complété</v>
       </c>
       <c r="G29" t="str">
-        <v>REQ-009</v>
+        <v>REQ-031</v>
       </c>
       <c r="H29" t="str">
-        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
+        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
       </c>
       <c r="I29" t="str">
-        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
+        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
       </c>
     </row>
     <row r="30">
@@ -1259,10 +1259,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C30" t="str">
-        <v>OpenAI optionnel</v>
+        <v>Modèle Ollama configurable</v>
       </c>
       <c r="D30" t="str">
-        <v>API key via .env, fallback auto Ollama si absent</v>
+        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
       </c>
       <c r="E30" t="str">
         <v>P1</v>
@@ -1271,13 +1271,13 @@
         <v>Complété</v>
       </c>
       <c r="G30" t="str">
-        <v>REQ-030</v>
+        <v>REQ-010</v>
       </c>
       <c r="H30" t="str">
-        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
+        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
       </c>
       <c r="I30" t="str">
-        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
+        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
       </c>
     </row>
     <row r="31">
@@ -1288,25 +1288,25 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C31" t="str">
-        <v>Thèmes personnalisés</v>
+        <v>OpenAI optionnel</v>
       </c>
       <c r="D31" t="str">
-        <v>Texte libre pour documents et questions</v>
+        <v>API key via .env, fallback auto Ollama si absent</v>
       </c>
       <c r="E31" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F31" t="str">
         <v>Complété</v>
       </c>
       <c r="G31" t="str">
-        <v>-</v>
+        <v>REQ-031</v>
       </c>
       <c r="H31" t="str">
-        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
+        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
       </c>
       <c r="I31" t="str">
-        <v>Permet flexibilité sur domaines audit custom</v>
+        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
       </c>
     </row>
     <row r="32">
@@ -1314,16 +1314,16 @@
         <v>REQ-031</v>
       </c>
       <c r="B32" t="str">
-        <v>Infrastructure &amp; Déploiement</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C32" t="str">
-        <v>Offline-first capability</v>
+        <v>Thèmes personnalisés</v>
       </c>
       <c r="D32" t="str">
-        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
+        <v>Texte libre pour documents et questions</v>
       </c>
       <c r="E32" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F32" t="str">
         <v>Complété</v>
@@ -1332,10 +1332,10 @@
         <v>-</v>
       </c>
       <c r="H32" t="str">
-        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
+        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
       </c>
       <c r="I32" t="str">
-        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
+        <v>Permet flexibilité sur domaines audit custom</v>
       </c>
     </row>
     <row r="33">
@@ -1346,25 +1346,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C33" t="str">
-        <v>Automation PowerShell</v>
+        <v>Offline-first capability</v>
       </c>
       <c r="D33" t="str">
-        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
+        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
       </c>
       <c r="E33" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F33" t="str">
         <v>Complété</v>
       </c>
       <c r="G33" t="str">
-        <v>REQ-028, REQ-031</v>
+        <v>-</v>
       </c>
       <c r="H33" t="str">
-        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
+        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
       </c>
       <c r="I33" t="str">
-        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
+        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
       </c>
     </row>
     <row r="34">
@@ -1375,25 +1375,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C34" t="str">
-        <v>Versionning Git &amp; GitHub</v>
+        <v>Automation PowerShell</v>
       </c>
       <c r="D34" t="str">
-        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
+        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
       </c>
       <c r="E34" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F34" t="str">
         <v>Complété</v>
       </c>
       <c r="G34" t="str">
-        <v>REQ-007, REQ-031</v>
+        <v>REQ-029, REQ-032</v>
       </c>
       <c r="H34" t="str">
-        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
+        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
       </c>
       <c r="I34" t="str">
-        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
+        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
       </c>
     </row>
     <row r="35">
@@ -1404,25 +1404,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C35" t="str">
-        <v>API REST Fastify</v>
+        <v>Versionning Git &amp; GitHub</v>
       </c>
       <c r="D35" t="str">
-        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
+        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
       </c>
       <c r="E35" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F35" t="str">
         <v>Complété</v>
       </c>
       <c r="G35" t="str">
-        <v>REQ-013, REQ-031</v>
+        <v>REQ-008, REQ-032</v>
       </c>
       <c r="H35" t="str">
-        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
+        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
       </c>
       <c r="I35" t="str">
-        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
+        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
       </c>
     </row>
     <row r="36">
@@ -1430,28 +1430,28 @@
         <v>REQ-035</v>
       </c>
       <c r="B36" t="str">
-        <v>UI/UX</v>
+        <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C36" t="str">
-        <v>UI React + TypeScript + Vite</v>
+        <v>API REST Fastify</v>
       </c>
       <c r="D36" t="str">
-        <v>Bundling optimisé, HMR dev mode</v>
+        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
       </c>
       <c r="E36" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F36" t="str">
         <v>Complété</v>
       </c>
       <c r="G36" t="str">
-        <v>REQ-017, REQ-031</v>
+        <v>REQ-014, REQ-032</v>
       </c>
       <c r="H36" t="str">
-        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
+        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
       </c>
       <c r="I36" t="str">
-        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
+        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
       </c>
     </row>
     <row r="37">
@@ -1462,10 +1462,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C37" t="str">
-        <v>Configuration IA section</v>
+        <v>UI React + TypeScript + Vite</v>
       </c>
       <c r="D37" t="str">
-        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
+        <v>Bundling optimisé, HMR dev mode</v>
       </c>
       <c r="E37" t="str">
         <v>P1</v>
@@ -1474,13 +1474,13 @@
         <v>Complété</v>
       </c>
       <c r="G37" t="str">
-        <v>REQ-024, REQ-031</v>
+        <v>REQ-018, REQ-032</v>
       </c>
       <c r="H37" t="str">
-        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
+        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
       </c>
       <c r="I37" t="str">
-        <v>UX: clair et accessible, pas scroll nécessaire</v>
+        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
       </c>
     </row>
     <row r="38">
@@ -1491,10 +1491,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C38" t="str">
-        <v>Génération questions section</v>
+        <v>Configuration IA section</v>
       </c>
       <c r="D38" t="str">
-        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
+        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
       </c>
       <c r="E38" t="str">
         <v>P1</v>
@@ -1503,13 +1503,13 @@
         <v>Complété</v>
       </c>
       <c r="G38" t="str">
-        <v>REQ-014, REQ-015, REQ-031</v>
+        <v>REQ-025, REQ-032</v>
       </c>
       <c r="H38" t="str">
-        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
+        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
       </c>
       <c r="I38" t="str">
-        <v>État uploadingReferential: loading indicator, disabled submit</v>
+        <v>UX: clair et accessible, pas scroll nécessaire</v>
       </c>
     </row>
     <row r="39">
@@ -1520,10 +1520,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C39" t="str">
-        <v>Référentiel documentaire section</v>
+        <v>Génération questions section</v>
       </c>
       <c r="D39" t="str">
-        <v>Ajouter document avec métas, liste affichée</v>
+        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
       </c>
       <c r="E39" t="str">
         <v>P1</v>
@@ -1532,13 +1532,13 @@
         <v>Complété</v>
       </c>
       <c r="G39" t="str">
-        <v>REQ-019, REQ-020, REQ-031</v>
+        <v>REQ-015, REQ-016, REQ-032</v>
       </c>
       <c r="H39" t="str">
-        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
+        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
       </c>
       <c r="I39" t="str">
-        <v>Erreurs affichées, success feedback, état documentS refresh</v>
+        <v>État uploadingReferential: loading indicator, disabled submit</v>
       </c>
     </row>
     <row r="40">
@@ -1549,10 +1549,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C40" t="str">
-        <v>Échelles métriques config</v>
+        <v>Référentiel documentaire section</v>
       </c>
       <c r="D40" t="str">
-        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
+        <v>Ajouter document avec métas, liste affichée</v>
       </c>
       <c r="E40" t="str">
         <v>P1</v>
@@ -1561,13 +1561,13 @@
         <v>Complété</v>
       </c>
       <c r="G40" t="str">
-        <v>REQ-021, REQ-022, REQ-031</v>
+        <v>REQ-020, REQ-021, REQ-032</v>
       </c>
       <c r="H40" t="str">
-        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
+        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
       </c>
       <c r="I40" t="str">
-        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
+        <v>Erreurs affichées, success feedback, état documentS refresh</v>
       </c>
     </row>
     <row r="41">
@@ -1578,10 +1578,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C41" t="str">
-        <v>Dashboard avec KPIs</v>
+        <v>Échelles métriques config</v>
       </c>
       <c r="D41" t="str">
-        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
+        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
       </c>
       <c r="E41" t="str">
         <v>P1</v>
@@ -1590,13 +1590,13 @@
         <v>Complété</v>
       </c>
       <c r="G41" t="str">
-        <v>-</v>
+        <v>REQ-022, REQ-023, REQ-032</v>
       </c>
       <c r="H41" t="str">
-        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
+        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
       </c>
       <c r="I41" t="str">
-        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
+        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
       </c>
     </row>
     <row r="42">
@@ -1607,10 +1607,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C42" t="str">
-        <v>Gestion entretiens</v>
+        <v>Dashboard avec KPIs</v>
       </c>
       <c r="D42" t="str">
-        <v>Interviewés, notes questions, scoring intégré</v>
+        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
       </c>
       <c r="E42" t="str">
         <v>P1</v>
@@ -1622,10 +1622,10 @@
         <v>-</v>
       </c>
       <c r="H42" t="str">
-        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
+        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
       </c>
       <c r="I42" t="str">
-        <v>Chaque note liée criterion + interviewee + score optionnel</v>
+        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
       </c>
     </row>
     <row r="43">
@@ -1636,10 +1636,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C43" t="str">
-        <v>Audit log viewer</v>
+        <v>Gestion entretiens</v>
       </c>
       <c r="D43" t="str">
-        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
+        <v>Interviewés, notes questions, scoring intégré</v>
       </c>
       <c r="E43" t="str">
         <v>P1</v>
@@ -1648,13 +1648,13 @@
         <v>Complété</v>
       </c>
       <c r="G43" t="str">
-        <v>REQ-041</v>
+        <v>-</v>
       </c>
       <c r="H43" t="str">
-        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
+        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
       </c>
       <c r="I43" t="str">
-        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
+        <v>Chaque note liée criterion + interviewee + score optionnel</v>
       </c>
     </row>
     <row r="44">
@@ -1665,25 +1665,25 @@
         <v>UI/UX</v>
       </c>
       <c r="C44" t="str">
-        <v>Export buttons</v>
+        <v>Audit log viewer</v>
       </c>
       <c r="D44" t="str">
-        <v>Boutons DOCX et CSV téléchargement</v>
+        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
       </c>
       <c r="E44" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F44" t="str">
         <v>Complété</v>
       </c>
       <c r="G44" t="str">
-        <v>-</v>
+        <v>REQ-042</v>
       </c>
       <c r="H44" t="str">
-        <v>POST /export-report et /export-csv. browser Blob download.</v>
+        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
       </c>
       <c r="I44" t="str">
-        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
       </c>
     </row>
     <row r="45">
@@ -1691,13 +1691,13 @@
         <v>REQ-044</v>
       </c>
       <c r="B45" t="str">
-        <v>Persévérance &amp; Facilité</v>
+        <v>UI/UX</v>
       </c>
       <c r="C45" t="str">
-        <v>Documentation complète</v>
+        <v>Export buttons</v>
       </c>
       <c r="D45" t="str">
-        <v>Setup guides, quickstart, git manual, examples références</v>
+        <v>Boutons DOCX et CSV téléchargement</v>
       </c>
       <c r="E45" t="str">
         <v>P2</v>
@@ -1709,13 +1709,13 @@
         <v>-</v>
       </c>
       <c r="H45" t="str">
-        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
+        <v>POST /export-report et /export-csv. browser Blob download.</v>
       </c>
       <c r="I45" t="str">
-        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
-      </c>
-    </row>
-    <row r="46" xml:space="preserve">
+        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+      </c>
+    </row>
+    <row r="46">
       <c r="A46" t="str">
         <v>REQ-045</v>
       </c>
@@ -1723,10 +1723,10 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C46" t="str">
-        <v>One-command installation</v>
+        <v>Documentation complète</v>
       </c>
       <c r="D46" t="str">
-        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+        <v>Setup guides, quickstart, git manual, examples références</v>
       </c>
       <c r="E46" t="str">
         <v>P2</v>
@@ -1737,12 +1737,11 @@
       <c r="G46" t="str">
         <v>-</v>
       </c>
-      <c r="H46" t="str" xml:space="preserve">
-        <v xml:space="preserve">.
- install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      <c r="H46" t="str">
+        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
       </c>
       <c r="I46" t="str">
-        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -1753,41 +1752,42 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C47" t="str">
+        <v>One-command installation</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+      </c>
+      <c r="E47" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G47" t="str">
+        <v>-</v>
+      </c>
+      <c r="H47" t="str" xml:space="preserve">
+        <v xml:space="preserve">.
+ install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      </c>
+      <c r="I47" t="str">
+        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
+        <v>REQ-047</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C48" t="str">
         <v>One-command launch</v>
       </c>
-      <c r="D47" t="str" xml:space="preserve">
+      <c r="D48" t="str" xml:space="preserve">
         <v xml:space="preserve">npm run dev ou .
 start-rubis.ps1 pour lancer tout</v>
       </c>
-      <c r="E47" t="str">
-        <v>P2</v>
-      </c>
-      <c r="F47" t="str">
-        <v>Complété</v>
-      </c>
-      <c r="G47" t="str">
-        <v>-</v>
-      </c>
-      <c r="H47" t="str">
-        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
-      </c>
-      <c r="I47" t="str">
-        <v>Détection auto erreurs, log output lisible</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>REQ-047</v>
-      </c>
-      <c r="B48" t="str">
-        <v>Persévérance &amp; Facilité</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Clear error messages</v>
-      </c>
-      <c r="D48" t="str">
-        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
-      </c>
       <c r="E48" t="str">
         <v>P2</v>
       </c>
@@ -1798,10 +1798,10 @@
         <v>-</v>
       </c>
       <c r="H48" t="str">
-        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
       </c>
       <c r="I48" t="str">
-        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+        <v>Détection auto erreurs, log output lisible</v>
       </c>
     </row>
     <row r="49">
@@ -1812,30 +1812,59 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C49" t="str">
-        <v>Roadmap versioning</v>
+        <v>Clear error messages</v>
       </c>
       <c r="D49" t="str">
-        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
       </c>
       <c r="E49" t="str">
         <v>P2</v>
       </c>
       <c r="F49" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G49" t="str">
         <v>-</v>
       </c>
       <c r="H49" t="str">
+        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>REQ-049</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Roadmap versioning</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+      </c>
+      <c r="E50" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Planifié</v>
+      </c>
+      <c r="G50" t="str">
+        <v>-</v>
+      </c>
+      <c r="H50" t="str">
         <v>Créer ROADMAP.xlsx avec specs, priorités, statuts, directives implémentation.</v>
       </c>
-      <c r="I49" t="str">
+      <c r="I50" t="str">
         <v>À committé dans git, mis à jour post-MVP pour v2 features</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I50"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: Add AI selection per phase in admin module to roadmap (REQ-012)
- New specification: Sélection IA par phase dans module admin
- Domain: Configuration & Flexibilité
- Priority: P1, Status: Planifié
- Feature: User can choose AI provider (OpenAI or Ollama) per audit workflow phase
- Implementation: Admin UI with phase config table, GET/POST /admin/ai-config endpoints
  Store in db.data.aiConfig: {phase, aiProvider, ollamaModel}
  Runtime routing: generateQuestions() checks active phase and routes to correct provider
- Use cases:
  * OpenAI for fast preparation phase (requires internet)
  * Ollama for offline field interviews
  * Mixed strategy per audit needs
- Validation: Check OPENAI_API_KEY if OpenAI selected
- Config scope: Per campaign or global
- Dependencies: REQ-004 (Admin module), REQ-009 (OpenAI), REQ-010 (Ollama), REQ-032 (API)
- Total: 50 specs (was 49)
- Updated dependency matrix: All IDs after REQ-011 shifted by +1
</commit_message>
<xml_diff>
--- a/ROADMAP.xlsx
+++ b/ROADMAP.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -763,28 +763,28 @@
         <v>REQ-012</v>
       </c>
       <c r="B13" t="str">
-        <v>IA &amp; Génération</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C13" t="str">
-        <v>Parsing référentiel multi-format</v>
+        <v>Sélection IA par phase dans module admin</v>
       </c>
       <c r="D13" t="str">
-        <v>Support PDF et Excel avec extraction de texte</v>
+        <v>Permet à l'utilisateur de choisir quelle IA utiliser (OpenAI ou Ollama) pour chaque phase du workflow d'audit via interface d'administration</v>
       </c>
       <c r="E13" t="str">
         <v>P1</v>
       </c>
       <c r="F13" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G13" t="str">
-        <v>REQ-008</v>
+        <v>REQ-004, REQ-009, REQ-010, REQ-031</v>
       </c>
       <c r="H13" t="str">
-        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
+        <v>Section admin protégée. Config par phase: {phase: '1.1-Préparation'|'1.2-Entretiens'|'1.3-Scoring'|'1.4-Rapports', aiProvider: 'openai'|'ollama', ollamaModel?: 'mistral'|'gemma3:4b'}. Endpoints: GET/POST /admin/ai-config. Stockage db.data.aiConfig. UI: table éditable avec dropdown provider + model. Au runtime, generateQuestions() check phase active et route vers bon provider.</v>
       </c>
       <c r="I13" t="str">
-        <v>Gère encodages UTF-8, caractères spéciaux</v>
+        <v>Flexibilité maximale: OpenAI rapide pour prépa, Ollama offline pour entretiens terrain. Validation: si OpenAI sélectionné, vérifier OPENAI_API_KEY présent. Config par campagne ou globale selon besoin.</v>
       </c>
     </row>
     <row r="14">
@@ -795,10 +795,10 @@
         <v>IA &amp; Génération</v>
       </c>
       <c r="C14" t="str">
-        <v>Prompt dynamique contextuel</v>
+        <v>Parsing référentiel multi-format</v>
       </c>
       <c r="D14" t="str">
-        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
+        <v>Support PDF et Excel avec extraction de texte</v>
       </c>
       <c r="E14" t="str">
         <v>P1</v>
@@ -810,10 +810,10 @@
         <v>REQ-008</v>
       </c>
       <c r="H14" t="str">
-        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
+        <v>parseReferentialFile() switch sur mimeType. pdf-parse pour PDF, xlsx pour Excel. Limiter 50KB.</v>
       </c>
       <c r="I14" t="str">
-        <v>Zod validation sur count (1-10), language (fr/en)</v>
+        <v>Gère encodages UTF-8, caractères spéciaux</v>
       </c>
     </row>
     <row r="15">
@@ -821,28 +821,28 @@
         <v>REQ-014</v>
       </c>
       <c r="B15" t="str">
-        <v>Structuration données</v>
+        <v>IA &amp; Génération</v>
       </c>
       <c r="C15" t="str">
-        <v>Modèle Document</v>
+        <v>Prompt dynamique contextuel</v>
       </c>
       <c r="D15" t="str">
-        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
+        <v>Criterion code/title, langue FR/EN, nombre questions 1-10</v>
       </c>
       <c r="E15" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F15" t="str">
         <v>Complété</v>
       </c>
       <c r="G15" t="str">
-        <v>REQ-002</v>
+        <v>REQ-008</v>
       </c>
       <c r="H15" t="str">
-        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
+        <v>openai.ts generateQuestionsFromReferential() construit userPrompt avec contexte injection</v>
       </c>
       <c r="I15" t="str">
-        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
+        <v>Zod validation sur count (1-10), language (fr/en)</v>
       </c>
     </row>
     <row r="16">
@@ -853,10 +853,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C16" t="str">
-        <v>Modèle Interviewé</v>
+        <v>Modèle Document</v>
       </c>
       <c r="D16" t="str">
-        <v>Nom complet, rôle, lié à campaign</v>
+        <v>Nom, thématique, version, date, sensibilité, résumé avec versioning</v>
       </c>
       <c r="E16" t="str">
         <v>P0</v>
@@ -868,10 +868,10 @@
         <v>REQ-002</v>
       </c>
       <c r="H16" t="str">
-        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
+        <v>db.data.documents: {id, campaignId, name, theme, version, date, sensitivity, summary}</v>
       </c>
       <c r="I16" t="str">
-        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
+        <v>Sensitivity enum: Public/Interne/Sensible/Confidentiel</v>
       </c>
     </row>
     <row r="17">
@@ -882,10 +882,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C17" t="str">
-        <v>Modèle Note d'entretien</v>
+        <v>Modèle Interviewé</v>
       </c>
       <c r="D17" t="str">
-        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
+        <v>Nom complet, rôle, lié à campaign</v>
       </c>
       <c r="E17" t="str">
         <v>P0</v>
@@ -894,13 +894,13 @@
         <v>Complété</v>
       </c>
       <c r="G17" t="str">
-        <v>REQ-005, REQ-015</v>
+        <v>REQ-002</v>
       </c>
       <c r="H17" t="str">
-        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
+        <v>db.data.interviewees: {id, campaignId, fullName, role}</v>
       </c>
       <c r="I17" t="str">
-        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
+        <v>Rôle texte libre (ex: RSSI, Directeur IT, etc.)</v>
       </c>
     </row>
     <row r="18">
@@ -911,25 +911,25 @@
         <v>Structuration données</v>
       </c>
       <c r="C18" t="str">
-        <v>Matrice de conformité</v>
+        <v>Modèle Note d'entretien</v>
       </c>
       <c r="D18" t="str">
-        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
+        <v>Contenu libre + scoring, lié à criterion et interviewé</v>
       </c>
       <c r="E18" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F18" t="str">
         <v>Complété</v>
       </c>
       <c r="G18" t="str">
-        <v>REQ-016</v>
+        <v>REQ-005, REQ-016</v>
       </c>
       <c r="H18" t="str">
-        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
+        <v>db.data.interviewNotes: {id, campaignId, criterionId, intervieweeId, content, score}</v>
       </c>
       <c r="I18" t="str">
-        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
+        <v>Score: 0-5 ou texte (conformité). Timestamp auto.</v>
       </c>
     </row>
     <row r="19">
@@ -940,10 +940,10 @@
         <v>Structuration données</v>
       </c>
       <c r="C19" t="str">
-        <v>Configuration Métriques</v>
+        <v>Matrice de conformité</v>
       </c>
       <c r="D19" t="str">
-        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
+        <v>Criterion code/title/theme, moyenne pondérée, questions répondues vs total</v>
       </c>
       <c r="E19" t="str">
         <v>P1</v>
@@ -952,13 +952,13 @@
         <v>Complété</v>
       </c>
       <c r="G19" t="str">
-        <v>REQ-002</v>
+        <v>REQ-017</v>
       </c>
       <c r="H19" t="str">
-        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
+        <v>Calculée à la volée depuis criterion + interviewNotes. GET /criteria/:campaignId aggregate.</v>
       </c>
       <c r="I19" t="str">
-        <v>Format texte (ex: '1-5') pour flexibilité</v>
+        <v>Poids configurable (voir Métriques). Moyenne excluant null/undefined.</v>
       </c>
     </row>
     <row r="20">
@@ -966,13 +966,13 @@
         <v>REQ-019</v>
       </c>
       <c r="B20" t="str">
-        <v>Audit &amp; Traçabilité</v>
+        <v>Structuration données</v>
       </c>
       <c r="C20" t="str">
-        <v>Audit Log complet</v>
+        <v>Configuration Métriques</v>
       </c>
       <c r="D20" t="str">
-        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
+        <v>Échelles personnalisables: Confidentialité, Intégrité, Disponibilité, Preuve</v>
       </c>
       <c r="E20" t="str">
         <v>P1</v>
@@ -981,13 +981,13 @@
         <v>Complété</v>
       </c>
       <c r="G20" t="str">
-        <v>REQ-002, REQ-031</v>
+        <v>REQ-002</v>
       </c>
       <c r="H20" t="str">
-        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
+        <v>POST /metric-scales. Stockage db.data.metricScales: {campaignId, confidentiality, integrity, availability, evidence}</v>
       </c>
       <c r="I20" t="str">
-        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
+        <v>Format texte (ex: '1-5') pour flexibilité</v>
       </c>
     </row>
     <row r="21">
@@ -998,10 +998,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C21" t="str">
-        <v>Filtrage logs par période</v>
+        <v>Audit Log complet</v>
       </c>
       <c r="D21" t="str">
-        <v>Vue 7j, 30j, tout (by date range filter)</v>
+        <v>Action, timestamp, détails, lié à campagne, stocker tous mouvements</v>
       </c>
       <c r="E21" t="str">
         <v>P1</v>
@@ -1010,13 +1010,13 @@
         <v>Complété</v>
       </c>
       <c r="G21" t="str">
-        <v>REQ-019</v>
+        <v>REQ-002, REQ-032</v>
       </c>
       <c r="H21" t="str">
-        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
+        <v>logAction(campaignId, action, details) helper. db.data.auditLogs array (reverse-chrono). Limit 2000 entrées.</v>
       </c>
       <c r="I21" t="str">
-        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
+        <v>Toutes mutations app tracées: campaign.created, criterion.created, etc.</v>
       </c>
     </row>
     <row r="22">
@@ -1027,10 +1027,10 @@
         <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C22" t="str">
-        <v>Filtrage logs par action</v>
+        <v>Filtrage logs par période</v>
       </c>
       <c r="D22" t="str">
-        <v>Filter sur type d'action (campaign.created, etc.)</v>
+        <v>Vue 7j, 30j, tout (by date range filter)</v>
       </c>
       <c r="E22" t="str">
         <v>P1</v>
@@ -1039,13 +1039,13 @@
         <v>Complété</v>
       </c>
       <c r="G22" t="str">
-        <v>REQ-019</v>
+        <v>REQ-020</v>
       </c>
       <c r="H22" t="str">
-        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
+        <v>GET /audit-log/:campaignId?period=7d|30d|all. Calcul date range côté backend.</v>
       </c>
       <c r="I22" t="str">
-        <v>Enum actions découvertes dynamiquement from logs</v>
+        <v>Filter UI: dropdown 3 options + affichage dynamique</v>
       </c>
     </row>
     <row r="23">
@@ -1053,28 +1053,28 @@
         <v>REQ-022</v>
       </c>
       <c r="B23" t="str">
-        <v>Rapports &amp; Exports</v>
+        <v>Audit &amp; Traçabilité</v>
       </c>
       <c r="C23" t="str">
-        <v>Export DOCX</v>
+        <v>Filtrage logs par action</v>
       </c>
       <c r="D23" t="str">
-        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
+        <v>Filter sur type d'action (campaign.created, etc.)</v>
       </c>
       <c r="E23" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F23" t="str">
         <v>Complété</v>
       </c>
       <c r="G23" t="str">
-        <v>REQ-007, REQ-017</v>
+        <v>REQ-020</v>
       </c>
       <c r="H23" t="str">
-        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
+        <v>GET /audit-log/:campaignId?action=all|campaign.created|etc. Sync action list UI.</v>
       </c>
       <c r="I23" t="str">
-        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
+        <v>Enum actions découvertes dynamiquement from logs</v>
       </c>
     </row>
     <row r="24">
@@ -1085,10 +1085,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C24" t="str">
-        <v>Export CSV</v>
+        <v>Export DOCX</v>
       </c>
       <c r="D24" t="str">
-        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
+        <v>Générer .docx avec questions, réponses, scoring, détails audit</v>
       </c>
       <c r="E24" t="str">
         <v>P2</v>
@@ -1097,13 +1097,13 @@
         <v>Complété</v>
       </c>
       <c r="G24" t="str">
-        <v>REQ-017, REQ-019</v>
+        <v>REQ-007, REQ-018</v>
       </c>
       <c r="H24" t="str">
-        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
+        <v>POST /export-report. Lib 'docx'. Génère paragraphes formatés + tableaux.</v>
       </c>
       <c r="I24" t="str">
-        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
+        <v>Téléchargement direct browser, nom: Rubis_Campaign_[date].docx</v>
       </c>
     </row>
     <row r="25">
@@ -1114,10 +1114,10 @@
         <v>Rapports &amp; Exports</v>
       </c>
       <c r="C25" t="str">
-        <v>Gestion des rapports</v>
+        <v>Export CSV</v>
       </c>
       <c r="D25" t="str">
-        <v>Stocker rapports générés avec titre, date gen, version</v>
+        <v>Audit logs + conformity matrix en CSV téléchargeable</v>
       </c>
       <c r="E25" t="str">
         <v>P2</v>
@@ -1126,13 +1126,13 @@
         <v>Complété</v>
       </c>
       <c r="G25" t="str">
-        <v>REQ-022, REQ-023</v>
+        <v>REQ-018, REQ-020</v>
       </c>
       <c r="H25" t="str">
-        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
+        <v>GET /export-csv/:campaignId. Convert array to CSV format. Headers: code,title,theme,conformity%</v>
       </c>
       <c r="I25" t="str">
-        <v>Récupérable dans UI, archivé pour traçabilité</v>
+        <v>2 fichiers: audit_logs.csv + conformity_matrix.csv</v>
       </c>
     </row>
     <row r="26">
@@ -1140,28 +1140,28 @@
         <v>REQ-025</v>
       </c>
       <c r="B26" t="str">
-        <v>Dashboard &amp; Visualisation</v>
+        <v>Rapports &amp; Exports</v>
       </c>
       <c r="C26" t="str">
-        <v>KPIs essentiels</v>
+        <v>Gestion des rapports</v>
       </c>
       <c r="D26" t="str">
-        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
+        <v>Stocker rapports générés avec titre, date gen, version</v>
       </c>
       <c r="E26" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F26" t="str">
         <v>Complété</v>
       </c>
       <c r="G26" t="str">
-        <v>REQ-014, REQ-015, REQ-016</v>
+        <v>REQ-023, REQ-024</v>
       </c>
       <c r="H26" t="str">
-        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
+        <v>db.data.auditReports: {id, campaignId, title, generatedAt, version, content}</v>
       </c>
       <c r="I26" t="str">
-        <v>Affiché en gros chiffres zone haute dashboard</v>
+        <v>Récupérable dans UI, archivé pour traçabilité</v>
       </c>
     </row>
     <row r="27">
@@ -1172,25 +1172,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C27" t="str">
-        <v>Matrice de conformité interactive</v>
+        <v>KPIs essentiels</v>
       </c>
       <c r="D27" t="str">
-        <v>Tableau avec % conformité par criterion, tri/filtre</v>
+        <v>Compteurs: documents, interviewés, notes, docs en attente, rapports, questions</v>
       </c>
       <c r="E27" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F27" t="str">
         <v>Complété</v>
       </c>
       <c r="G27" t="str">
-        <v>REQ-017</v>
+        <v>REQ-015, REQ-016, REQ-017</v>
       </c>
       <c r="H27" t="str">
-        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
+        <v>GET /dashboard-kpis/:campaignId. Aggregate counts depuis db.data.*</v>
       </c>
       <c r="I27" t="str">
-        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
+        <v>Affiché en gros chiffres zone haute dashboard</v>
       </c>
     </row>
     <row r="28">
@@ -1201,25 +1201,25 @@
         <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C28" t="str">
-        <v>Graphiques optionnels (futur)</v>
+        <v>Matrice de conformité interactive</v>
       </c>
       <c r="D28" t="str">
-        <v>Tendances audit timeline, pie charts conformity domains</v>
+        <v>Tableau avec % conformité par criterion, tri/filtre</v>
       </c>
       <c r="E28" t="str">
-        <v>P3</v>
+        <v>P2</v>
       </c>
       <c r="F28" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G28" t="str">
-        <v>REQ-025</v>
+        <v>REQ-018</v>
       </c>
       <c r="H28" t="str">
-        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
+        <v>Affichage table React. Données GET /criteria/:campaignId. Tri sur weighting, answeredQuestions.</v>
       </c>
       <c r="I28" t="str">
-        <v>MVP n'a pas graphiques, architecture prête pour.</v>
+        <v>Couleurs: rouge &lt;50%, orange 50-80%, vert &gt;80%</v>
       </c>
     </row>
     <row r="29">
@@ -1227,28 +1227,28 @@
         <v>REQ-028</v>
       </c>
       <c r="B29" t="str">
-        <v>Configuration &amp; Flexibilité</v>
+        <v>Dashboard &amp; Visualisation</v>
       </c>
       <c r="C29" t="str">
-        <v>Support multilingue</v>
+        <v>Graphiques optionnels (futur)</v>
       </c>
       <c r="D29" t="str">
-        <v>FR et EN, sélection par campaign</v>
+        <v>Tendances audit timeline, pie charts conformity domains</v>
       </c>
       <c r="E29" t="str">
-        <v>P1</v>
+        <v>P3</v>
       </c>
       <c r="F29" t="str">
-        <v>Complété</v>
+        <v>Planifié</v>
       </c>
       <c r="G29" t="str">
-        <v>REQ-031</v>
+        <v>REQ-026</v>
       </c>
       <c r="H29" t="str">
-        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
+        <v>Ajouter recharts ou Chart.js si requis. Endpoints déjà supportent data.</v>
       </c>
       <c r="I29" t="str">
-        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
+        <v>MVP n'a pas graphiques, architecture prête pour.</v>
       </c>
     </row>
     <row r="30">
@@ -1259,10 +1259,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C30" t="str">
-        <v>Modèle Ollama configurable</v>
+        <v>Support multilingue</v>
       </c>
       <c r="D30" t="str">
-        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
+        <v>FR et EN, sélection par campaign</v>
       </c>
       <c r="E30" t="str">
         <v>P1</v>
@@ -1271,13 +1271,13 @@
         <v>Complété</v>
       </c>
       <c r="G30" t="str">
-        <v>REQ-010</v>
+        <v>REQ-032</v>
       </c>
       <c r="H30" t="str">
-        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
+        <v>POST /campaigns body.language enum 'fr'|'en'. Stocké campaign. UI affiche langue active.</v>
       </c>
       <c r="I30" t="str">
-        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
+        <v>Prompts IA adaptent langue dynamiquement (français si campaign.language=fr)</v>
       </c>
     </row>
     <row r="31">
@@ -1288,10 +1288,10 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C31" t="str">
-        <v>OpenAI optionnel</v>
+        <v>Modèle Ollama configurable</v>
       </c>
       <c r="D31" t="str">
-        <v>API key via .env, fallback auto Ollama si absent</v>
+        <v>Switcher mistral ou gemma3:4b sans redémarrage</v>
       </c>
       <c r="E31" t="str">
         <v>P1</v>
@@ -1300,13 +1300,13 @@
         <v>Complété</v>
       </c>
       <c r="G31" t="str">
-        <v>REQ-031</v>
+        <v>REQ-010</v>
       </c>
       <c r="H31" t="str">
-        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
+        <v>GET/POST /config. État currentOllamaModel runtime. Boutons UI permutent.</v>
       </c>
       <c r="I31" t="str">
-        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
+        <v>Persist pas en DB (runtime only). Config peut sauver .env si demandé.</v>
       </c>
     </row>
     <row r="32">
@@ -1317,25 +1317,25 @@
         <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C32" t="str">
-        <v>Thèmes personnalisés</v>
+        <v>OpenAI optionnel</v>
       </c>
       <c r="D32" t="str">
-        <v>Texte libre pour documents et questions</v>
+        <v>API key via .env, fallback auto Ollama si absent</v>
       </c>
       <c r="E32" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F32" t="str">
         <v>Complété</v>
       </c>
       <c r="G32" t="str">
-        <v>-</v>
+        <v>REQ-032</v>
       </c>
       <c r="H32" t="str">
-        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
+        <v>OPENAI_API_KEY=... in .env.example. openai.ts check process.env, instantiate si présent.</v>
       </c>
       <c r="I32" t="str">
-        <v>Permet flexibilité sur domaines audit custom</v>
+        <v>generateQuestionsFromOpenAI() try-catch, log warn si clé manquante</v>
       </c>
     </row>
     <row r="33">
@@ -1343,16 +1343,16 @@
         <v>REQ-032</v>
       </c>
       <c r="B33" t="str">
-        <v>Infrastructure &amp; Déploiement</v>
+        <v>Configuration &amp; Flexibilité</v>
       </c>
       <c r="C33" t="str">
-        <v>Offline-first capability</v>
+        <v>Thèmes personnalisés</v>
       </c>
       <c r="D33" t="str">
-        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
+        <v>Texte libre pour documents et questions</v>
       </c>
       <c r="E33" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F33" t="str">
         <v>Complété</v>
@@ -1361,10 +1361,10 @@
         <v>-</v>
       </c>
       <c r="H33" t="str">
-        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
+        <v>document.theme et question.theme: string (no enum). UI input texte libre.</v>
       </c>
       <c r="I33" t="str">
-        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
+        <v>Permet flexibilité sur domaines audit custom</v>
       </c>
     </row>
     <row r="34">
@@ -1375,25 +1375,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C34" t="str">
-        <v>Automation PowerShell</v>
+        <v>Offline-first capability</v>
       </c>
       <c r="D34" t="str">
-        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
+        <v>Aucune dépendance cloud obligatoire, Ollama local suffisant</v>
       </c>
       <c r="E34" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F34" t="str">
         <v>Complété</v>
       </c>
       <c r="G34" t="str">
-        <v>REQ-029, REQ-032</v>
+        <v>-</v>
       </c>
       <c r="H34" t="str">
-        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
+        <v>Ollama localhost:11434 défaut. OpenAI optionnel. DB lowdb fichier local.</v>
       </c>
       <c r="I34" t="str">
-        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
+        <v>Testé sur HP EliteBook Ryzen 5 8540U, 15GB RAM, 138GB disk</v>
       </c>
     </row>
     <row r="35">
@@ -1404,25 +1404,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C35" t="str">
-        <v>Versionning Git &amp; GitHub</v>
+        <v>Automation PowerShell</v>
       </c>
       <c r="D35" t="str">
-        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
+        <v>Scripts install-ollama, start-rubis, compare-models pour non-techniques</v>
       </c>
       <c r="E35" t="str">
-        <v>P1</v>
+        <v>P2</v>
       </c>
       <c r="F35" t="str">
         <v>Complété</v>
       </c>
       <c r="G35" t="str">
-        <v>REQ-008, REQ-032</v>
+        <v>REQ-030, REQ-033</v>
       </c>
       <c r="H35" t="str">
-        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
+        <v>Fichiers: install-ollama.ps1, start-rubis.ps1, compare-ollama-models.ps1 root repo</v>
       </c>
       <c r="I35" t="str">
-        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
+        <v>Chaque script &gt;=70 lines, logs détaillés, exit codes corrects</v>
       </c>
     </row>
     <row r="36">
@@ -1433,25 +1433,25 @@
         <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C36" t="str">
-        <v>API REST Fastify</v>
+        <v>Versionning Git &amp; GitHub</v>
       </c>
       <c r="D36" t="str">
-        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
+        <v>Repository github.com/emi5650/Rubis, SSH auth, 54 commits initiaux</v>
       </c>
       <c r="E36" t="str">
-        <v>P0</v>
+        <v>P1</v>
       </c>
       <c r="F36" t="str">
         <v>Complété</v>
       </c>
       <c r="G36" t="str">
-        <v>REQ-014, REQ-032</v>
+        <v>REQ-008, REQ-033</v>
       </c>
       <c r="H36" t="str">
-        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
+        <v>.gitignore configué. Push via SSH Ed25519 key. GitHub repo créé.</v>
       </c>
       <c r="I36" t="str">
-        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
+        <v>SSH key generé + configuré. Prêt pour CI/CD futur.</v>
       </c>
     </row>
     <row r="37">
@@ -1459,28 +1459,28 @@
         <v>REQ-036</v>
       </c>
       <c r="B37" t="str">
-        <v>UI/UX</v>
+        <v>Infrastructure &amp; Déploiement</v>
       </c>
       <c r="C37" t="str">
-        <v>UI React + TypeScript + Vite</v>
+        <v>API REST Fastify</v>
       </c>
       <c r="D37" t="str">
-        <v>Bundling optimisé, HMR dev mode</v>
+        <v>Framework web API 5.x, CORS enabled, multipart upload 50MB limit</v>
       </c>
       <c r="E37" t="str">
-        <v>P1</v>
+        <v>P0</v>
       </c>
       <c r="F37" t="str">
         <v>Complété</v>
       </c>
       <c r="G37" t="str">
-        <v>REQ-018, REQ-032</v>
+        <v>REQ-015, REQ-033</v>
       </c>
       <c r="H37" t="str">
-        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
+        <v>Fastify app.ts. @fastify/cors registered. @fastify/multipart 9.0.1</v>
       </c>
       <c r="I37" t="str">
-        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
+        <v>Écoute 0.0.0.0:4000 pour accès réseau local</v>
       </c>
     </row>
     <row r="38">
@@ -1491,10 +1491,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C38" t="str">
-        <v>Configuration IA section</v>
+        <v>UI React + TypeScript + Vite</v>
       </c>
       <c r="D38" t="str">
-        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
+        <v>Bundling optimisé, HMR dev mode</v>
       </c>
       <c r="E38" t="str">
         <v>P1</v>
@@ -1503,13 +1503,13 @@
         <v>Complété</v>
       </c>
       <c r="G38" t="str">
-        <v>REQ-025, REQ-032</v>
+        <v>REQ-019, REQ-033</v>
       </c>
       <c r="H38" t="str">
-        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
+        <v>Apps/web/src/App.tsx. Vite config. 29 modules bundled.</v>
       </c>
       <c r="I38" t="str">
-        <v>UX: clair et accessible, pas scroll nécessaire</v>
+        <v>Production build: 229KB JS gzip, 1.17KB CSS gzip</v>
       </c>
     </row>
     <row r="39">
@@ -1520,10 +1520,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C39" t="str">
-        <v>Génération questions section</v>
+        <v>Configuration IA section</v>
       </c>
       <c r="D39" t="str">
-        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
+        <v>Boutons model switching mistral/gemma3:4b avec statut visuel</v>
       </c>
       <c r="E39" t="str">
         <v>P1</v>
@@ -1532,13 +1532,13 @@
         <v>Complété</v>
       </c>
       <c r="G39" t="str">
-        <v>REQ-015, REQ-016, REQ-032</v>
+        <v>REQ-026, REQ-033</v>
       </c>
       <c r="H39" t="str">
-        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
+        <v>Section card en haut App.tsx. Boutons onClick switchOllamaModel(). Vert si actif.</v>
       </c>
       <c r="I39" t="str">
-        <v>État uploadingReferential: loading indicator, disabled submit</v>
+        <v>UX: clair et accessible, pas scroll nécessaire</v>
       </c>
     </row>
     <row r="40">
@@ -1549,10 +1549,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C40" t="str">
-        <v>Référentiel documentaire section</v>
+        <v>Génération questions section</v>
       </c>
       <c r="D40" t="str">
-        <v>Ajouter document avec métas, liste affichée</v>
+        <v>Upload fichier, select count, bouton 'Générer via IA', affichage résultat</v>
       </c>
       <c r="E40" t="str">
         <v>P1</v>
@@ -1561,13 +1561,13 @@
         <v>Complété</v>
       </c>
       <c r="G40" t="str">
-        <v>REQ-020, REQ-021, REQ-032</v>
+        <v>REQ-016, REQ-017, REQ-033</v>
       </c>
       <c r="H40" t="str">
-        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
+        <v>Form &lt;input type=file accept=.pdf,.xlsx&gt;. Input number 1-10. Submitter disabled si !criterionId</v>
       </c>
       <c r="I40" t="str">
-        <v>Erreurs affichées, success feedback, état documentS refresh</v>
+        <v>État uploadingReferential: loading indicator, disabled submit</v>
       </c>
     </row>
     <row r="41">
@@ -1578,10 +1578,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C41" t="str">
-        <v>Échelles métriques config</v>
+        <v>Référentiel documentaire section</v>
       </c>
       <c r="D41" t="str">
-        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
+        <v>Ajouter document avec métas, liste affichée</v>
       </c>
       <c r="E41" t="str">
         <v>P1</v>
@@ -1590,13 +1590,13 @@
         <v>Complété</v>
       </c>
       <c r="G41" t="str">
-        <v>REQ-022, REQ-023, REQ-032</v>
+        <v>REQ-021, REQ-022, REQ-033</v>
       </c>
       <c r="H41" t="str">
-        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
+        <v>Form: name, theme, version, date, sensitivity select, summary. POST /documents</v>
       </c>
       <c r="I41" t="str">
-        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
+        <v>Erreurs affichées, success feedback, état documentS refresh</v>
       </c>
     </row>
     <row r="42">
@@ -1607,10 +1607,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C42" t="str">
-        <v>Dashboard avec KPIs</v>
+        <v>Échelles métriques config</v>
       </c>
       <c r="D42" t="str">
-        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
+        <v>Input pour Confidentialité, Intégrité, Disponibilité, Preuve (ex: 1-5)</v>
       </c>
       <c r="E42" t="str">
         <v>P1</v>
@@ -1619,13 +1619,13 @@
         <v>Complété</v>
       </c>
       <c r="G42" t="str">
-        <v>-</v>
+        <v>REQ-023, REQ-024, REQ-033</v>
       </c>
       <c r="H42" t="str">
-        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
+        <v>Form 4 inputs texte. POST /metric-scales. Sauvé par campaign.</v>
       </c>
       <c r="I42" t="str">
-        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
+        <v>Format libre permet audit custom (ex: YES/NO ou 0-10)</v>
       </c>
     </row>
     <row r="43">
@@ -1636,10 +1636,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C43" t="str">
-        <v>Gestion entretiens</v>
+        <v>Dashboard avec KPIs</v>
       </c>
       <c r="D43" t="str">
-        <v>Interviewés, notes questions, scoring intégré</v>
+        <v>Affichage cards avec compteurs, matrice conformité, audit log viewer</v>
       </c>
       <c r="E43" t="str">
         <v>P1</v>
@@ -1651,10 +1651,10 @@
         <v>-</v>
       </c>
       <c r="H43" t="str">
-        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
+        <v>useState dashboardKpis, matrixDetails. GET /dashboard-kpis. Render grid cards.</v>
       </c>
       <c r="I43" t="str">
-        <v>Chaque note liée criterion + interviewee + score optionnel</v>
+        <v>View mode 'dashboard' toggle TOP (workspace vs dashboard)</v>
       </c>
     </row>
     <row r="44">
@@ -1665,10 +1665,10 @@
         <v>UI/UX</v>
       </c>
       <c r="C44" t="str">
-        <v>Audit log viewer</v>
+        <v>Gestion entretiens</v>
       </c>
       <c r="D44" t="str">
-        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
+        <v>Interviewés, notes questions, scoring intégré</v>
       </c>
       <c r="E44" t="str">
         <v>P1</v>
@@ -1677,13 +1677,13 @@
         <v>Complété</v>
       </c>
       <c r="G44" t="str">
-        <v>REQ-042</v>
+        <v>-</v>
       </c>
       <c r="H44" t="str">
-        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
+        <v>Sections: Ajouter interviewé form. Notes d'entretien table. Scoring form.</v>
       </c>
       <c r="I44" t="str">
-        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
+        <v>Chaque note liée criterion + interviewee + score optionnel</v>
       </c>
     </row>
     <row r="45">
@@ -1694,25 +1694,25 @@
         <v>UI/UX</v>
       </c>
       <c r="C45" t="str">
-        <v>Export buttons</v>
+        <v>Audit log viewer</v>
       </c>
       <c r="D45" t="str">
-        <v>Boutons DOCX et CSV téléchargement</v>
+        <v>Tableau logs avec filtres période (7d/30d/all) et action</v>
       </c>
       <c r="E45" t="str">
-        <v>P2</v>
+        <v>P1</v>
       </c>
       <c r="F45" t="str">
         <v>Complété</v>
       </c>
       <c r="G45" t="str">
-        <v>-</v>
+        <v>REQ-043</v>
       </c>
       <c r="H45" t="str">
-        <v>POST /export-report et /export-csv. browser Blob download.</v>
+        <v>Dropdowns: period, action filter. GET /audit-log avec query params. Table affiche action/timestamp/details</v>
       </c>
       <c r="I45" t="str">
-        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+        <v>Sync knownActions dynamiquement depuis logs récupérés</v>
       </c>
     </row>
     <row r="46">
@@ -1720,13 +1720,13 @@
         <v>REQ-045</v>
       </c>
       <c r="B46" t="str">
-        <v>Persévérance &amp; Facilité</v>
+        <v>UI/UX</v>
       </c>
       <c r="C46" t="str">
-        <v>Documentation complète</v>
+        <v>Export buttons</v>
       </c>
       <c r="D46" t="str">
-        <v>Setup guides, quickstart, git manual, examples références</v>
+        <v>Boutons DOCX et CSV téléchargement</v>
       </c>
       <c r="E46" t="str">
         <v>P2</v>
@@ -1738,13 +1738,13 @@
         <v>-</v>
       </c>
       <c r="H46" t="str">
-        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
+        <v>POST /export-report et /export-csv. browser Blob download.</v>
       </c>
       <c r="I46" t="str">
-        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
-      </c>
-    </row>
-    <row r="47" xml:space="preserve">
+        <v>Noms fichiers: Rubis_Campaign_[date]_[format]</v>
+      </c>
+    </row>
+    <row r="47">
       <c r="A47" t="str">
         <v>REQ-046</v>
       </c>
@@ -1752,10 +1752,10 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C47" t="str">
-        <v>One-command installation</v>
+        <v>Documentation complète</v>
       </c>
       <c r="D47" t="str">
-        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+        <v>Setup guides, quickstart, git manual, examples références</v>
       </c>
       <c r="E47" t="str">
         <v>P2</v>
@@ -1766,12 +1766,11 @@
       <c r="G47" t="str">
         <v>-</v>
       </c>
-      <c r="H47" t="str" xml:space="preserve">
-        <v xml:space="preserve">.
- install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      <c r="H47" t="str">
+        <v>Fichiers: SETUP_OLLAMA.md, SETUP_OPENAI.md, GETTING_STARTED.md, QUICKSTART.md, README.md, GIT_MANUAL_INSTRUCTIONS.md</v>
       </c>
       <c r="I47" t="str">
-        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+        <v>&gt;1500 lines docs. Français + English mix selon besoin.</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -1782,41 +1781,42 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C48" t="str">
+        <v>One-command installation</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Non-tech user peut installer Rubis complet en 1 commande</v>
+      </c>
+      <c r="E48" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Complété</v>
+      </c>
+      <c r="G48" t="str">
+        <v>-</v>
+      </c>
+      <c r="H48" t="str" xml:space="preserve">
+        <v xml:space="preserve">.
+ install-ollama.ps1 détecte, installe Ollama, download Mistral, setup env.</v>
+      </c>
+      <c r="I48" t="str">
+        <v>~30min première fois (download 2.3GB Mistral). ~5min après.</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
+        <v>REQ-048</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C49" t="str">
         <v>One-command launch</v>
       </c>
-      <c r="D48" t="str" xml:space="preserve">
+      <c r="D49" t="str" xml:space="preserve">
         <v xml:space="preserve">npm run dev ou .
 start-rubis.ps1 pour lancer tout</v>
       </c>
-      <c r="E48" t="str">
-        <v>P2</v>
-      </c>
-      <c r="F48" t="str">
-        <v>Complété</v>
-      </c>
-      <c r="G48" t="str">
-        <v>-</v>
-      </c>
-      <c r="H48" t="str">
-        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
-      </c>
-      <c r="I48" t="str">
-        <v>Détection auto erreurs, log output lisible</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>REQ-048</v>
-      </c>
-      <c r="B49" t="str">
-        <v>Persévérance &amp; Facilité</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Clear error messages</v>
-      </c>
-      <c r="D49" t="str">
-        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
-      </c>
       <c r="E49" t="str">
         <v>P2</v>
       </c>
@@ -1827,10 +1827,10 @@
         <v>-</v>
       </c>
       <c r="H49" t="str">
-        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+        <v>start-rubis.ps1: verify Ollama, launch Ollama bg terminal, npm run dev. ~30 sec.</v>
       </c>
       <c r="I49" t="str">
-        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+        <v>Détection auto erreurs, log output lisible</v>
       </c>
     </row>
     <row r="50">
@@ -1841,30 +1841,59 @@
         <v>Persévérance &amp; Facilité</v>
       </c>
       <c r="C50" t="str">
-        <v>Roadmap versioning</v>
+        <v>Clear error messages</v>
       </c>
       <c r="D50" t="str">
-        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+        <v>UI affiche erreurs compréhensibles, logs API détaillés</v>
       </c>
       <c r="E50" t="str">
         <v>P2</v>
       </c>
       <c r="F50" t="str">
-        <v>Planifié</v>
+        <v>Complété</v>
       </c>
       <c r="G50" t="str">
         <v>-</v>
       </c>
       <c r="H50" t="str">
+        <v>UI setErrorMessage(). API log.error(). Try-catch tous endpoints.</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Users voient actionable feedback (ex: 'Modèle Ollama non trouvé, essayez gemma3:4b')</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>REQ-050</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Persévérance &amp; Facilité</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Roadmap versioning</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Fichier Excel roadmap dans repo pour futur maintenance/sprints</v>
+      </c>
+      <c r="E51" t="str">
+        <v>P2</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Planifié</v>
+      </c>
+      <c r="G51" t="str">
+        <v>-</v>
+      </c>
+      <c r="H51" t="str">
         <v>Créer ROADMAP.xlsx avec specs, priorités, statuts, directives implémentation.</v>
       </c>
-      <c r="I50" t="str">
+      <c r="I51" t="str">
         <v>À committé dans git, mis à jour post-MVP pour v2 features</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I50"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I51"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>